<commit_message>
Move X reasons to last remark column; fill unlisted XS blade info from other sellers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -609,8 +609,8 @@
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -666,12 +666,12 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>공용 키날 비고</t>
+          <t>판매 페이지</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>판매 페이지</t>
+          <t>비고 (공용 키날 X 사유)</t>
         </is>
       </c>
     </row>
@@ -724,16 +724,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 2Buttons XKB508EN</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L2" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -784,14 +780,14 @@
           <t>Xhorse VVDI Key Tool Garage Style Wired Remote Control, 2Buttons XKGD12EN</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>차고문 리모컨</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -844,16 +840,12 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Flip Remote, 2Buttons XKTO01EN</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -904,14 +896,14 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Key Head Remote, 2Buttons, TOY43 XKTO05EN</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>키날 포함 제품 (TOY43 고정)</t>
-        </is>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -964,16 +956,12 @@
           <t>Xhorse VVDI Key Tool Audi Style Wired Flip Remote, 3Buttons XKA600EN</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1024,16 +1012,12 @@
           <t>Xhorse VVDI Key Tool Audi Style Wired Flip Remote, 3Buttons XKAU01EN</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1084,16 +1068,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 3Buttons XKB501EN</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1144,16 +1124,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 3Buttons Blue XKB503EN</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1204,16 +1180,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 3Buttons Green XKB504EN</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L10" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1264,16 +1236,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 3Buttons Orange XKB505EN</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L11" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1324,16 +1292,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 3Buttons XKB506EN</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L12" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1384,16 +1348,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 3Buttons XKB510EN</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L13" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1444,16 +1404,12 @@
           <t>Xhorse VVDI Key Tool Buick Style Wired Flip Remote, 3Buttons XKBU03EN</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L14" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1504,16 +1460,12 @@
           <t>Xhorse VVDI Key Tool Peugeot Citroen Style Wired Flip Remote, 3Buttons XKDS00EN</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1560,14 +1512,14 @@
           <t>Xhorse VVDI Key Tool Wired Remote Control, 3Buttons XKFEF1EN Red</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L16" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -1616,14 +1568,14 @@
           <t>Xhorse VVDI Key Tool Wired Remote Control, 3Buttons XKFEF5EN</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L17" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -1676,16 +1628,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 3Buttons XKGA83EN</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L18" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1736,16 +1684,12 @@
           <t>Xhorse VVDI Key Tool Honda Style Wired Flip Remote, 3Buttons XKHO00EN</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L19" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1796,16 +1740,12 @@
           <t>Xhorse VVDI Key Tool Honda Style Wired Flip Remote, 3Buttons XKHO02EN</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L20" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1856,14 +1796,14 @@
           <t>Xhorse VVDI Key Tool Hyundai Kia Style Wired Remote, 3Buttons XKHY00EN</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L21" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -1916,16 +1856,12 @@
           <t>Xhorse VVDI Key Tool Hyundai Kia Style Wired Flip Remote, 3Buttons XKHY02EN</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L22" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1976,16 +1912,12 @@
           <t>Xhorse VVDI Key Tool Hyundai Style Wired Flip Remote, 3Buttons XKHY05EN</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L23" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2036,16 +1968,12 @@
           <t>Xhorse VVDI Key Tool Bmw Style Wired Flip Remote, 3Buttons XKKF02EN</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L24" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2096,16 +2024,12 @@
           <t>Xhorse VVDI Key Tool Bmw Style Wired Remote, 3Buttons XKKF03EN</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L25" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2156,16 +2080,12 @@
           <t>Xhorse VVDI Key Tool Bmw Style Wired Remote, 3Buttons XKKF21EN</t>
         </is>
       </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L26" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2216,16 +2136,12 @@
           <t>Xhorse VVDI Key Tool Bmw Style Wired Flip Remote, 3Buttons XKKF23EN</t>
         </is>
       </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L27" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2276,16 +2192,12 @@
           <t>Xhorse VVDI Key Tool Lexus Style Wired Flip Remote, 3Buttons XKLEX0EN</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L28" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2336,16 +2248,12 @@
           <t>Xhorse VVDI Key Tool Lexus Style Wired Remote, 3Buttons XKLKS0EN</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L29" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2396,16 +2304,12 @@
           <t>Xhorse VVDI Key Tool Mazda Style Wired Flip Remote, 3Buttons XKMA00EN</t>
         </is>
       </c>
-      <c r="K30" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L30" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2456,16 +2360,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Wired Flip Remote, 3Buttons XKMQB1EN</t>
         </is>
       </c>
-      <c r="K31" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L31" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2516,16 +2416,12 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Flip Remote, 3Buttons XKTO00EN</t>
         </is>
       </c>
-      <c r="K32" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L32" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2576,14 +2472,14 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Key Head Remote, 3Buttons, TOY43 XKTO03EN</t>
         </is>
       </c>
-      <c r="K33" s="5" t="inlineStr">
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
         <is>
           <t>키날 포함 제품 (TOY43 고정)</t>
-        </is>
-      </c>
-      <c r="L33" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -2636,14 +2532,14 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Key Head Remote, 3Buttons, TOY43 XKTO04EN</t>
         </is>
       </c>
-      <c r="K34" s="5" t="inlineStr">
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
         <is>
           <t>키날 포함 제품 (TOY43 고정)</t>
-        </is>
-      </c>
-      <c r="L34" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -2696,16 +2592,12 @@
           <t>Xhorse VVDI Key Tool Audi Style Wired Flip Remote, 4Buttons XKAU02EN</t>
         </is>
       </c>
-      <c r="K35" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L35" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2756,16 +2648,12 @@
           <t>Xhorse VVDI Key Tool GM Style Wired Flip Remote, 4Buttons XKBU01EN</t>
         </is>
       </c>
-      <c r="K36" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L36" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2816,16 +2704,12 @@
           <t>Xhorse VVDI Key Tool Buick Style Wired Flip Remote, 4Buttons XKBU02EN</t>
         </is>
       </c>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L37" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2876,16 +2760,12 @@
           <t>Xhorse VVDI Key Tool Cadillac Style Wired Flip Remote, 4Buttons XKCD02EN</t>
         </is>
       </c>
-      <c r="K38" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L38" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2932,14 +2812,14 @@
           <t>Xhorse VVDI Key Tool Wired Remote Control, 4Buttons XKFEF2EN Red</t>
         </is>
       </c>
-      <c r="K39" s="5" t="inlineStr">
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L39" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -2988,14 +2868,14 @@
           <t>Xhorse VVDI Key Tool Wired Remote Control, 4Buttons XKFEF6EN</t>
         </is>
       </c>
-      <c r="K40" s="5" t="inlineStr">
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L40" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3048,16 +2928,12 @@
           <t>Xhorse VVDI Key Tool Ford Style Wired Flip Remote, 4Buttons XKFO01EN</t>
         </is>
       </c>
-      <c r="K41" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L41" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3108,14 +2984,14 @@
           <t>Xhorse VVDI Key Tool Ford Style Wired Remote Control, 4Buttons XKFO02EN</t>
         </is>
       </c>
-      <c r="K42" s="5" t="inlineStr">
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L42" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3164,14 +3040,14 @@
           <t>Xhorse VVDI Key Tool Wired Remote Control, 4Buttons XKGD10EN</t>
         </is>
       </c>
-      <c r="K43" s="5" t="inlineStr">
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L43" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3224,14 +3100,14 @@
           <t>Xhorse VVDI Key Tool Garage Style Wired Remote Control, 4Buttons XKGHG1EN</t>
         </is>
       </c>
-      <c r="K44" s="5" t="inlineStr">
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
         <is>
           <t>차고문 리모컨</t>
-        </is>
-      </c>
-      <c r="L44" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3284,16 +3160,12 @@
           <t>Xhorse VVDI Key Tool Honda Style Wired Flip Remote, 4Buttons XKHO01EN</t>
         </is>
       </c>
-      <c r="K45" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L45" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3344,14 +3216,14 @@
           <t>Xhorse VVDI Key Tool Hyundai Kia Style Wired Remote Control, 4Buttons XKHY01EN</t>
         </is>
       </c>
-      <c r="K46" s="5" t="inlineStr">
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L46" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3404,14 +3276,14 @@
           <t>Xhorse VVDI Key Tool Hyundai Style Wired Remote Control, 4Buttons XKHY04EN</t>
         </is>
       </c>
-      <c r="K47" s="5" t="inlineStr">
+      <c r="K47" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L47" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3464,16 +3336,12 @@
           <t>Xhorse VVDI Key Tool Knife Style Wired Flip Remote, 4Buttons XKKF20EN</t>
         </is>
       </c>
-      <c r="K48" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L48" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3524,16 +3392,12 @@
           <t>Xhorse VVDI Key Tool Knife Style Wired Flip Remote, 4Buttons XKM800EN</t>
         </is>
       </c>
-      <c r="K49" s="5" t="inlineStr">
-        <is>
-          <t>폴딩키 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L49" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K49" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3584,14 +3448,14 @@
           <t>Xhorse VVDI Key Tool Nissan Style Wired Remote Control, 4Buttons XKNI00EN</t>
         </is>
       </c>
-      <c r="K50" s="5" t="inlineStr">
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L50" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3644,14 +3508,14 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Key Head Remote, 4Buttons, TOY43 XKTO02EN</t>
         </is>
       </c>
-      <c r="K51" s="5" t="inlineStr">
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
         <is>
           <t>키날 포함 제품 (TOY43 고정)</t>
-        </is>
-      </c>
-      <c r="L51" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3704,14 +3568,14 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Key Head Remote, 4Buttons, TOY43 XKTO06EN</t>
         </is>
       </c>
-      <c r="K52" s="5" t="inlineStr">
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
         <is>
           <t>키날 포함 제품 (TOY43 고정)</t>
-        </is>
-      </c>
-      <c r="L52" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3764,16 +3628,12 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Flip Remote, 4Buttons XKTO10EN</t>
         </is>
       </c>
-      <c r="K53" s="5" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L53" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K53" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3820,14 +3680,14 @@
           <t>Xhorse VVDI Key Tool Wired Remote Control, 4Buttons XKXH00EN</t>
         </is>
       </c>
-      <c r="K54" s="5" t="inlineStr">
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L54" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L54" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3876,14 +3736,14 @@
           <t>Xhorse VVDI Key Tool Wired Remote Control, 4Buttons Blue XKXH01EN</t>
         </is>
       </c>
-      <c r="K55" s="5" t="inlineStr">
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L55" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3932,14 +3792,14 @@
           <t>Xhorse VVDI Key Tool Golden Wired Remote Control, 4Buttons XKXH02EN</t>
         </is>
       </c>
-      <c r="K56" s="5" t="inlineStr">
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L56" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L56" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -3988,14 +3848,14 @@
           <t>Xhorse VVDI Key Tool Wired Remote Control, 4Buttons XKXH03EN</t>
         </is>
       </c>
-      <c r="K57" s="5" t="inlineStr">
+      <c r="K57" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L57" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -4044,14 +3904,14 @@
           <t>Xhorse VVDI Key Tool Blue Wired Remote Control, 4Buttons XKXH04EN</t>
         </is>
       </c>
-      <c r="K58" s="5" t="inlineStr">
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L58" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L58" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -4100,14 +3960,14 @@
           <t>Xhorse VVDI Key Tool Golden Wired Remote Control, 4Buttons XKXH05EN</t>
         </is>
       </c>
-      <c r="K59" s="5" t="inlineStr">
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L59" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -4160,14 +4020,14 @@
           <t>Xhorse VVDI Key Tool Honda Style Wired Remote Control, 5Buttons XKHO03EN</t>
         </is>
       </c>
-      <c r="K60" s="5" t="inlineStr">
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L60" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L60" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -4220,14 +4080,14 @@
           <t>Xhorse VVDI Key Tool Honda Style Wired Remote Control, 5Buttons XKHO04EN</t>
         </is>
       </c>
-      <c r="K61" s="5" t="inlineStr">
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L61" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -4280,14 +4140,14 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wired Remote Control, 5Buttons XKTO08EN</t>
         </is>
       </c>
-      <c r="K62" s="5" t="inlineStr">
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L62" s="5" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L62" s="7" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -4340,14 +4200,14 @@
           <t>Xhorse VVDI Key Tool Suzuki Style Wireless Remote Key, 2Buttons XNSZ01EN</t>
         </is>
       </c>
-      <c r="K63" s="12" t="inlineStr">
+      <c r="K63" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L63" s="12" t="inlineStr">
         <is>
           <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
-        </is>
-      </c>
-      <c r="L63" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -4400,16 +4260,12 @@
           <t>Xhorse VVDI Key Tool Audi Style Wireless Flip Remote, 3Buttons XNAU01EN</t>
         </is>
       </c>
-      <c r="K64" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L64" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K64" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L64" s="12" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
@@ -4460,16 +4316,12 @@
           <t>Xhorse VVDI Key Tool Peugeot Citroen Style Wireless Flip Remote, 3Buttons XNDS00EN</t>
         </is>
       </c>
-      <c r="K65" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L65" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K65" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L65" s="12" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
@@ -4520,16 +4372,12 @@
           <t>Xhorse VVDI Key Tool Honda Style Wireless Flip Remote, 3Buttons XNHO00EN</t>
         </is>
       </c>
-      <c r="K66" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L66" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K66" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L66" s="12" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
@@ -4580,16 +4428,12 @@
           <t>Xhorse VVDI Key Tool Hyundai Kia Style Wireless Flip Remote, 3Buttons XNHY02EN</t>
         </is>
       </c>
-      <c r="K67" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L67" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K67" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L67" s="12" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
@@ -4640,16 +4484,12 @@
           <t>Xhorse VVDI Key Tool Hyundai Style Wireless Remote Key, 3Buttons XNHY04EN</t>
         </is>
       </c>
-      <c r="K68" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L68" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K68" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L68" s="12" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
@@ -4700,16 +4540,12 @@
           <t>Xhorse VVDI Key Tool Toyota Style Wireless Flip Remote, 3Buttons XNTO00EN</t>
         </is>
       </c>
-      <c r="K69" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L69" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K69" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L69" s="12" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
@@ -4760,16 +4596,12 @@
           <t>Xhorse VVDI Key Tool Audi Style Wireless Flip Remote, 4Buttons XNAU02EN</t>
         </is>
       </c>
-      <c r="K70" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L70" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K70" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L70" s="12" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
@@ -4820,16 +4652,12 @@
           <t>Xhorse VVDI Key Tool GM Style Wireless Flip Remote, 4Buttons XNBU01EN</t>
         </is>
       </c>
-      <c r="K71" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L71" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K71" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L71" s="12" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
@@ -4880,16 +4708,12 @@
           <t>Xhorse VVDI Key Tool Ford Style Wireless Flip Remote, 4Buttons XNFO01EN</t>
         </is>
       </c>
-      <c r="K72" s="12" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L72" s="14" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K72" s="14" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L72" s="12" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
@@ -4940,16 +4764,12 @@
           <t>Xhorse VVDI Key Tool Peugeot Citroen Style Super Remote, 3Buttons XT27 Super Chip XEDS01EN</t>
         </is>
       </c>
-      <c r="K73" s="19" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L73" s="21" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K73" s="21" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L73" s="19" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
@@ -5000,16 +4820,12 @@
           <t>Xhorse VVDI Key Tool Knife Style Super Remote, 3Buttons, XT27 Super Chip XEKF21EN</t>
         </is>
       </c>
-      <c r="K74" s="19" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L74" s="21" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K74" s="21" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L74" s="19" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="16" t="inlineStr">
@@ -5060,16 +4876,12 @@
           <t>Xhorse VVDI Key Tool Lexus Style Super Remote, 3Buttons, XT27 Super Chip XELEX0EN</t>
         </is>
       </c>
-      <c r="K75" s="19" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L75" s="21" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K75" s="21" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L75" s="19" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="16" t="inlineStr">
@@ -5120,16 +4932,12 @@
           <t>Xhorse VVDI Key Tool Volkswagen Style Super Remote, 3Buttons, XT27 Super Chip XEMQB1EN</t>
         </is>
       </c>
-      <c r="K76" s="19" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L76" s="21" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K76" s="21" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L76" s="19" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
@@ -5180,16 +4988,12 @@
           <t>Xhorse VVDI Key Tool Toyota Style Super Remote, 3Buttons, XT27 Super Chip XETO00EN</t>
         </is>
       </c>
-      <c r="K77" s="19" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L77" s="21" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K77" s="21" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L77" s="19" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="16" t="inlineStr">
@@ -5240,16 +5044,12 @@
           <t>Xhorse VVDI Key Tool Ford Style Super Remote, 4Buttons, XT27 Super Chip XEFO01EN</t>
         </is>
       </c>
-      <c r="K78" s="19" t="inlineStr">
-        <is>
-          <t>판매처가 공용 키날을 옵션으로 지정</t>
-        </is>
-      </c>
-      <c r="L78" s="21" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K78" s="21" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L78" s="19" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="22" t="inlineStr">
@@ -5300,14 +5100,14 @@
           <t>Xhorse Bmw Motorcycle Smart Key XSBMM0GL XM38 2Buttons</t>
         </is>
       </c>
-      <c r="K79" s="25" t="inlineStr">
+      <c r="K79" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L79" s="25" t="inlineStr">
         <is>
           <t>키날 포함 제품</t>
-        </is>
-      </c>
-      <c r="L79" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5360,14 +5160,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 2Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K80" s="25" t="inlineStr">
+      <c r="K80" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L80" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L80" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5420,14 +5220,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 2Buttons+Panic XSTO01EN</t>
         </is>
       </c>
-      <c r="K81" s="25" t="inlineStr">
+      <c r="K81" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L81" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L81" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5480,14 +5280,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 2Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K82" s="25" t="inlineStr">
+      <c r="K82" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L82" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L82" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5540,14 +5340,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 2Buttons+Panic XSTO01EN</t>
         </is>
       </c>
-      <c r="K83" s="25" t="inlineStr">
+      <c r="K83" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L83" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L83" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5600,14 +5400,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 2Buttons+Panic XSTO01EN</t>
         </is>
       </c>
-      <c r="K84" s="25" t="inlineStr">
+      <c r="K84" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L84" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L84" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5660,14 +5460,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 2Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K85" s="25" t="inlineStr">
+      <c r="K85" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L85" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L85" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5720,14 +5520,14 @@
           <t>Xhorse Lexus Smart Key 315/433MHz 2Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K86" s="25" t="inlineStr">
+      <c r="K86" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L86" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L86" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5780,16 +5580,12 @@
           <t>Xhorse Universal Smart Key XSKF01EN BMW Style 3Buttons</t>
         </is>
       </c>
-      <c r="K87" s="25" t="inlineStr">
-        <is>
-          <t>판매처가 공용 폴딩 키날을 지정</t>
-        </is>
-      </c>
-      <c r="L87" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K87" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L87" s="25" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="22" t="inlineStr">
@@ -5840,16 +5636,12 @@
           <t>Xhorse Universal Smart Key XSKFF1EN Knife Style 3Buttons</t>
         </is>
       </c>
-      <c r="K88" s="25" t="inlineStr">
-        <is>
-          <t>판매처가 공용 폴딩 키날을 지정</t>
-        </is>
-      </c>
-      <c r="L88" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K88" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L88" s="25" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="22" t="inlineStr">
@@ -5900,14 +5692,14 @@
           <t>Xhorse XSMA41EN Smart Key Board With 3Buttons for Audi MLB Cars</t>
         </is>
       </c>
-      <c r="K89" s="25" t="inlineStr">
+      <c r="K89" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L89" s="25" t="inlineStr">
         <is>
           <t>아우디·포르쉐 HU162 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L89" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -5960,14 +5752,14 @@
           <t>Xhorse XSMA4YEN Smart Key Board With 3Buttons for Audi A4 MLB Cars Works with Xhorse MLB Tool</t>
         </is>
       </c>
-      <c r="K90" s="25" t="inlineStr">
+      <c r="K90" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L90" s="25" t="inlineStr">
         <is>
           <t>아우디·포르쉐 HU162 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L90" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6020,14 +5812,14 @@
           <t>Xhorse XSMA8YEN Smart Key Board With 3Buttons for Audi A8 MLB Cars Works with Xhorse MLB Tool</t>
         </is>
       </c>
-      <c r="K91" s="25" t="inlineStr">
+      <c r="K91" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L91" s="25" t="inlineStr">
         <is>
           <t>아우디·포르쉐 HU162 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L91" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6080,14 +5872,14 @@
           <t>Xhorse XSMPSYEN Smart Key Board With 3Buttons for Porsche MLB Cars Works with Xhorse MLB Tool</t>
         </is>
       </c>
-      <c r="K92" s="25" t="inlineStr">
+      <c r="K92" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L92" s="25" t="inlineStr">
         <is>
           <t>아우디·포르쉐 HU162 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L92" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6140,16 +5932,12 @@
           <t>Xhorse Universal Smart Key XSMQB1EN VW MQB Style 3Buttons</t>
         </is>
       </c>
-      <c r="K93" s="25" t="inlineStr">
-        <is>
-          <t>판매처가 공용 폴딩 키날을 지정</t>
-        </is>
-      </c>
-      <c r="L93" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K93" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L93" s="25" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="22" t="inlineStr">
@@ -6200,16 +5988,12 @@
           <t>Xhorse Universal Smart Key XSSC01EN Supercar Style Marble Black Color XM38 3Buttons</t>
         </is>
       </c>
-      <c r="K94" s="25" t="inlineStr">
-        <is>
-          <t>XM38 범용. 판매처가 공용 폴딩 키날 구매 안내</t>
-        </is>
-      </c>
-      <c r="L94" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K94" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L94" s="25" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="22" t="inlineStr">
@@ -6260,16 +6044,12 @@
           <t>Xhorse Universal Smart Key XSSC04EN Supercar Style Miami Blue Color XM38 3Buttons</t>
         </is>
       </c>
-      <c r="K95" s="25" t="inlineStr">
-        <is>
-          <t>XM38 범용. 판매처가 공용 폴딩 키날 구매 안내</t>
-        </is>
-      </c>
-      <c r="L95" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K95" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L95" s="25" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="22" t="inlineStr">
@@ -6320,16 +6100,12 @@
           <t>Xhorse Universal Smart Key XSSC05EN Supercar Style Marble Grey Color XM38 3Buttons</t>
         </is>
       </c>
-      <c r="K96" s="25" t="inlineStr">
-        <is>
-          <t>XM38 범용. 판매처가 공용 폴딩 키날 구매 안내</t>
-        </is>
-      </c>
-      <c r="L96" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K96" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L96" s="25" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="22" t="inlineStr">
@@ -6380,14 +6156,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K97" s="25" t="inlineStr">
+      <c r="K97" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L97" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L97" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6440,14 +6216,14 @@
           <t>Xhorse Lexus Smart Key 315/433MHz 3Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K98" s="25" t="inlineStr">
+      <c r="K98" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L98" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L98" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6500,14 +6276,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K99" s="25" t="inlineStr">
+      <c r="K99" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L99" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L99" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6560,14 +6336,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K100" s="25" t="inlineStr">
+      <c r="K100" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L100" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L100" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6620,14 +6396,14 @@
           <t>Xhorse Universal Smart Key For Audi 315MHz 433MHz 868MHz 4Buttons XSADJ1EN</t>
         </is>
       </c>
-      <c r="K101" s="25" t="inlineStr">
-        <is>
-          <t>판매처 미기재 (확인 필요)</t>
-        </is>
-      </c>
-      <c r="L101" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
+      <c r="K101" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L101" s="25" t="inlineStr">
+        <is>
+          <t>UHS: 기판만 판매(Board only), 비상키 미포함. 아우디 A4·A5·A6·A7·A8·Q5 (2008~2016) 순정형 쉘에 넣는 기판 → 해당 쉘용 비상키 필요</t>
         </is>
       </c>
     </row>
@@ -6680,14 +6456,14 @@
           <t>Xhorse XSBMB1EN BMW Smart Key PCB BMW Bread Style for F/G Chassis BDC2 BDC3 4Buttons</t>
         </is>
       </c>
-      <c r="K102" s="25" t="inlineStr">
+      <c r="K102" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L102" s="25" t="inlineStr">
         <is>
           <t>기판만 판매. 쉘에 맞는 비상키 필요</t>
-        </is>
-      </c>
-      <c r="L102" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6740,14 +6516,14 @@
           <t>Xhorse XSBMU1EN BMW Smart Key PCB BMW U Style for F/G Chassis BDC2 BDC3 4Buttons</t>
         </is>
       </c>
-      <c r="K103" s="25" t="inlineStr">
+      <c r="K103" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L103" s="25" t="inlineStr">
         <is>
           <t>기판만 판매. 쉘에 맞는 비상키 필요</t>
-        </is>
-      </c>
-      <c r="L103" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -6800,16 +6576,12 @@
           <t>Xhorse Universal Smart Key XSCH01EN Chrysler Style XM38 4Buttons</t>
         </is>
       </c>
-      <c r="K104" s="25" t="inlineStr">
-        <is>
-          <t>판매처가 공용 폴딩 키날을 지정</t>
-        </is>
-      </c>
-      <c r="L104" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K104" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L104" s="25" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="22" t="inlineStr">
@@ -6837,9 +6609,9 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F105" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F105" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G105" s="22" t="inlineStr">
@@ -6860,16 +6632,12 @@
           <t>Xhorse Universal Smart Key XSCL01EN Chevrolet Style 4Buttons</t>
         </is>
       </c>
-      <c r="K105" s="25" t="inlineStr">
-        <is>
-          <t>판매처 미기재 (확인 필요)</t>
-        </is>
-      </c>
-      <c r="L105" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K105" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L105" s="25" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="22" t="inlineStr">
@@ -6920,16 +6688,12 @@
           <t>Xhorse Universal Smart Key XSCS00EN Hyundai Style 4Buttons</t>
         </is>
       </c>
-      <c r="K106" s="25" t="inlineStr">
-        <is>
-          <t>판매처가 공용 폴딩 키날을 지정</t>
-        </is>
-      </c>
-      <c r="L106" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K106" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L106" s="25" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="22" t="inlineStr">
@@ -6957,9 +6721,9 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F107" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F107" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G107" s="22" t="inlineStr">
@@ -6980,16 +6744,12 @@
           <t>Xhorse Universal Smart Key XSDFX2EN Knife Style 4Buttons</t>
         </is>
       </c>
-      <c r="K107" s="25" t="inlineStr">
-        <is>
-          <t>판매처 미기재 (확인 필요)</t>
-        </is>
-      </c>
-      <c r="L107" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K107" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L107" s="25" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="22" t="inlineStr">
@@ -7040,16 +6800,12 @@
           <t>Xhorse Universal Smart Key XSFO02EN Ford Style XM38 4Buttons</t>
         </is>
       </c>
-      <c r="K108" s="25" t="inlineStr">
-        <is>
-          <t>XM38 범용. 판매처가 공용 폴딩 키날 구매 안내</t>
-        </is>
-      </c>
-      <c r="L108" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K108" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L108" s="25" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="22" t="inlineStr">
@@ -7100,16 +6856,12 @@
           <t>Xhorse Universal Smart Key XSGA80EN VW Style XM38 4Buttons</t>
         </is>
       </c>
-      <c r="K109" s="25" t="inlineStr">
-        <is>
-          <t>XM38 범용. 판매처가 공용 폴딩 키날 구매 안내</t>
-        </is>
-      </c>
-      <c r="L109" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K109" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L109" s="25" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="22" t="inlineStr">
@@ -7156,14 +6908,14 @@
           <t>Xhorse King Card Slimmest Universal Smart Key 4Buttons XSKC04EN Diamond Blue Colour</t>
         </is>
       </c>
-      <c r="K110" s="25" t="inlineStr">
+      <c r="K110" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L110" s="25" t="inlineStr">
         <is>
           <t>키날 없는 제품</t>
-        </is>
-      </c>
-      <c r="L110" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -7212,14 +6964,14 @@
           <t>Xhorse King Card Slimmest Universal Smart Key 4Buttons XSKC05EN Sky Blue Colour</t>
         </is>
       </c>
-      <c r="K111" s="25" t="inlineStr">
+      <c r="K111" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L111" s="25" t="inlineStr">
         <is>
           <t>키날 없는 제품</t>
-        </is>
-      </c>
-      <c r="L111" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -7272,16 +7024,12 @@
           <t>Xhorse Universal Smart Key XSKF20EN BMW Style 4Buttons</t>
         </is>
       </c>
-      <c r="K112" s="25" t="inlineStr">
-        <is>
-          <t>판매처가 공용 폴딩 키날을 지정</t>
-        </is>
-      </c>
-      <c r="L112" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K112" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L112" s="25" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="22" t="inlineStr">
@@ -7332,16 +7080,12 @@
           <t>Xhorse Universal Smart Key XSKF21EN BMW Style 4Buttons</t>
         </is>
       </c>
-      <c r="K113" s="25" t="inlineStr">
-        <is>
-          <t>판매처가 공용 폴딩 키날을 지정</t>
-        </is>
-      </c>
-      <c r="L113" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K113" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L113" s="25" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="22" t="inlineStr">
@@ -7392,16 +7136,12 @@
           <t>Xhorse Universal Smart Key XSKF30EN Knife Style 4Buttons</t>
         </is>
       </c>
-      <c r="K114" s="25" t="inlineStr">
-        <is>
-          <t>판매처가 공용 폴딩 키날을 지정</t>
-        </is>
-      </c>
-      <c r="L114" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K114" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L114" s="25" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="22" t="inlineStr">
@@ -7429,9 +7169,9 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F115" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F115" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G115" s="22" t="inlineStr">
@@ -7452,16 +7192,12 @@
           <t>Xhorse Universal Smart Key XSKFF0EN Knife Style 4Buttons</t>
         </is>
       </c>
-      <c r="K115" s="25" t="inlineStr">
-        <is>
-          <t>판매처 미기재 (확인 필요)</t>
-        </is>
-      </c>
-      <c r="L115" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K115" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L115" s="25" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="22" t="inlineStr">
@@ -7512,14 +7248,14 @@
           <t>Xhorse Universal Smart Key XSNIS2EN Nissan Style 4Buttons</t>
         </is>
       </c>
-      <c r="K116" s="25" t="inlineStr">
+      <c r="K116" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L116" s="25" t="inlineStr">
         <is>
           <t>닛산 NSN14 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L116" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -7572,16 +7308,12 @@
           <t>Xhorse Universal Smart Key XSPS01EN Porsche Style XM38 4Buttons Red</t>
         </is>
       </c>
-      <c r="K117" s="25" t="inlineStr">
-        <is>
-          <t>XM38 범용. 판매처가 공용 폴딩 키날 구매 안내</t>
-        </is>
-      </c>
-      <c r="L117" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K117" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L117" s="25" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="22" t="inlineStr">
@@ -7632,16 +7364,12 @@
           <t>Xhorse Universal Smart Key XSSBR0EN Subaru Style XM38 4Buttons</t>
         </is>
       </c>
-      <c r="K118" s="25" t="inlineStr">
-        <is>
-          <t>XM38 범용. 판매처가 공용 폴딩 키날 구매 안내</t>
-        </is>
-      </c>
-      <c r="L118" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K118" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L118" s="25" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="22" t="inlineStr">
@@ -7692,14 +7420,14 @@
           <t>Xhorse Toyota XM38 Smart Key 4Buttons Support 4D 8A 4A All in One With Key Shell XSTO01EN</t>
         </is>
       </c>
-      <c r="K119" s="25" t="inlineStr">
+      <c r="K119" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L119" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L119" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -7752,14 +7480,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons SUV XSTO01EN</t>
         </is>
       </c>
-      <c r="K120" s="25" t="inlineStr">
+      <c r="K120" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L120" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L120" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -7812,14 +7540,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K121" s="25" t="inlineStr">
+      <c r="K121" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L121" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L121" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -7872,14 +7600,14 @@
           <t>Xhorse Lexus Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K122" s="25" t="inlineStr">
+      <c r="K122" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L122" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L122" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -7932,14 +7660,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K123" s="25" t="inlineStr">
+      <c r="K123" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L123" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L123" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -7992,14 +7720,14 @@
           <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K124" s="25" t="inlineStr">
+      <c r="K124" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L124" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L124" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8052,14 +7780,14 @@
           <t>Xhorse Lexus Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
-      <c r="K125" s="25" t="inlineStr">
+      <c r="K125" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L125" s="25" t="inlineStr">
         <is>
           <t>토요타·렉서스 TOY48 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L125" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8112,14 +7840,14 @@
           <t>Xhorse Universal Smart Key XSTO03EN Toyota Style XM38 4Buttons</t>
         </is>
       </c>
-      <c r="K126" s="25" t="inlineStr">
-        <is>
-          <t>판매처 미기재 (확인 필요)</t>
-        </is>
-      </c>
-      <c r="L126" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
+      <c r="K126" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L126" s="25" t="inlineStr">
+        <is>
+          <t>판매처 간 상충: key4는 공용 폴딩 키날 안내, 같은 XM38 토요타형(XSTO01EN)은 ABKEYS가 TOY48 전용 비상키 지정 → 구매 전 확인 필요</t>
         </is>
       </c>
     </row>
@@ -8172,16 +7900,12 @@
           <t>Xhorse Universal Smart Key XSCD01EN Cadillac Style XM38 5Buttons</t>
         </is>
       </c>
-      <c r="K127" s="25" t="inlineStr">
-        <is>
-          <t>XM38 범용. 판매처가 공용 폴딩 키날 구매 안내</t>
-        </is>
-      </c>
-      <c r="L127" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+      <c r="K127" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L127" s="25" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="22" t="inlineStr">
@@ -8232,14 +7956,14 @@
           <t>Xhorse Universal Smart Key XSJP01EN Jeep Style XM38 5Buttons</t>
         </is>
       </c>
-      <c r="K128" s="25" t="inlineStr">
+      <c r="K128" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L128" s="25" t="inlineStr">
         <is>
           <t>키날 포함 제품</t>
-        </is>
-      </c>
-      <c r="L128" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8292,14 +8016,14 @@
           <t>Xhorse Universal Smart Key XSLR01EN Land Rover Style XM38 5Buttons</t>
         </is>
       </c>
-      <c r="K129" s="25" t="inlineStr">
-        <is>
-          <t>랜드로버 HU101 전용 비상키</t>
-        </is>
-      </c>
-      <c r="L129" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
+      <c r="K129" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L129" s="25" t="inlineStr">
+        <is>
+          <t>ABKEYS가 랜드로버 HU101 전용 스마트키 비상키 지정 (key4는 공용 폴딩 키날 안내 → 판매처 간 상충)</t>
         </is>
       </c>
     </row>
@@ -8352,14 +8076,14 @@
           <t>Xhorse Universal Smart Key XSLR03EN Land Rover Style For NXP Chip 5Buttons</t>
         </is>
       </c>
-      <c r="K130" s="25" t="inlineStr">
-        <is>
-          <t>판매처 미기재 (확인 필요)</t>
-        </is>
-      </c>
-      <c r="L130" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
+      <c r="K130" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L130" s="25" t="inlineStr">
+        <is>
+          <t>Locksmith Keyless 등 다른 판매처도 키날 정보 없음. 같은 랜드로버형 XSLR01EN은 HU101 전용 비상키 지정 → 확인 필요</t>
         </is>
       </c>
     </row>
@@ -8408,14 +8132,14 @@
           <t>Xhorse Bluetooth Digital Smart Key XSBTK0EN Supports iOS Android - Turn your Phone to a Car Key</t>
         </is>
       </c>
-      <c r="K131" s="25" t="inlineStr">
+      <c r="K131" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L131" s="25" t="inlineStr">
         <is>
           <t>키날 없는 제품</t>
-        </is>
-      </c>
-      <c r="L131" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8464,14 +8188,14 @@
           <t>Xhorse Smart Watch Wearable Super Car Key Midnight Black SW-007 XSWK02EN</t>
         </is>
       </c>
-      <c r="K132" s="25" t="inlineStr">
+      <c r="K132" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L132" s="25" t="inlineStr">
         <is>
           <t>키날 없는 제품</t>
-        </is>
-      </c>
-      <c r="L132" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8520,14 +8244,14 @@
           <t>Xhorse Smart Watch Wearable Super Car Key Navy Blue SW-007 XSWK05EN</t>
         </is>
       </c>
-      <c r="K133" s="25" t="inlineStr">
+      <c r="K133" s="27" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L133" s="25" t="inlineStr">
         <is>
           <t>키날 없는 제품</t>
-        </is>
-      </c>
-      <c r="L133" s="27" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8580,14 +8304,14 @@
           <t>Xhorse Universal Smart Key PCB XZBT42EN Honda Style 2Buttons</t>
         </is>
       </c>
-      <c r="K134" s="32" t="inlineStr">
+      <c r="K134" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L134" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L134" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8640,14 +8364,14 @@
           <t>Xhorse XZADM1EN Special Remote Board With XT27B Chip &amp; 3Buttons For Audi MQB48 Models</t>
         </is>
       </c>
-      <c r="K135" s="32" t="inlineStr">
+      <c r="K135" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L135" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L135" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8700,14 +8424,14 @@
           <t>Xhorse Universal Smart Key PCB XZBT41EN Honda Style 3Buttons</t>
         </is>
       </c>
-      <c r="K136" s="32" t="inlineStr">
+      <c r="K136" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L136" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L136" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8760,14 +8484,14 @@
           <t>Xhorse XZBTM1EN Special Smart Key Board With 3Buttons for Honda Motorcycles</t>
         </is>
       </c>
-      <c r="K137" s="32" t="inlineStr">
+      <c r="K137" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L137" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L137" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8820,14 +8544,14 @@
           <t>Xhorse XZKA81EN Special Smart Key Board With 3Buttons for Hyundai &amp; Kia Cars</t>
         </is>
       </c>
-      <c r="K138" s="32" t="inlineStr">
+      <c r="K138" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L138" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L138" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8880,14 +8604,14 @@
           <t>Xhorse XZKA83EN Special Smart Key Board With 3Buttons for Hyundai &amp; Kia Cars</t>
         </is>
       </c>
-      <c r="K139" s="32" t="inlineStr">
+      <c r="K139" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L139" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L139" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -8940,14 +8664,14 @@
           <t>Xhorse XZKA84EN Special Smart Key Board With 3Buttons for Hyundai Cars</t>
         </is>
       </c>
-      <c r="K140" s="32" t="inlineStr">
+      <c r="K140" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L140" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L140" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -9000,14 +8724,14 @@
           <t>Xhorse XZMZD6EN Special Smart Key Board With 3Buttons for Mazda Cars</t>
         </is>
       </c>
-      <c r="K141" s="32" t="inlineStr">
+      <c r="K141" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L141" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L141" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -9060,14 +8784,14 @@
           <t>Xhorse XZPG00EN Special Smart Key Board With 3Buttons for Peugeot &amp; Citroen Cars</t>
         </is>
       </c>
-      <c r="K142" s="32" t="inlineStr">
+      <c r="K142" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L142" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L142" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -9120,14 +8844,14 @@
           <t>Xhorse XZVGM1EN Special Remote Board With XT27B Chip &amp; 3Buttons For Volkswagen MQB48 Models</t>
         </is>
       </c>
-      <c r="K143" s="32" t="inlineStr">
+      <c r="K143" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L143" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L143" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -9180,14 +8904,14 @@
           <t>Xhorse Universal Smart Key PCB XZBT40EN Honda Style 4Buttons</t>
         </is>
       </c>
-      <c r="K144" s="32" t="inlineStr">
+      <c r="K144" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L144" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L144" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -9240,14 +8964,14 @@
           <t>Xhorse Universal Smart Key PCB XZBT43EN Honda Style 4Buttons</t>
         </is>
       </c>
-      <c r="K145" s="32" t="inlineStr">
+      <c r="K145" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L145" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L145" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -9300,14 +9024,14 @@
           <t>Xhorse XZBT51EN Special Smart Key Board With 4Buttons for Honda Cars</t>
         </is>
       </c>
-      <c r="K146" s="32" t="inlineStr">
+      <c r="K146" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L146" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L146" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -9360,14 +9084,14 @@
           <t>Xhorse XZKA82EN Special Smart Key Board With 4Buttons for Hyundai &amp; Kia Cars</t>
         </is>
       </c>
-      <c r="K147" s="32" t="inlineStr">
+      <c r="K147" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L147" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L147" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
@@ -9420,167 +9144,167 @@
           <t>Xhorse Universal Smart Key PCB XZBT44EN Honda Style 5Buttons</t>
         </is>
       </c>
-      <c r="K148" s="32" t="inlineStr">
+      <c r="K148" s="34" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="L148" s="32" t="inlineStr">
         <is>
           <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
-        </is>
-      </c>
-      <c r="L148" s="34" t="inlineStr">
-        <is>
-          <t>링크</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L148"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L87" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L90" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L91" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L92" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L93" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L94" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L98" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L99" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L107" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L108" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L109" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L110" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L111" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L112" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L113" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L114" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L115" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L116" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L117" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L118" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L119" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L123" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L124" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L128" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L132" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L133" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L137" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L138" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L139" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L141" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L142" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L143" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L144" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L145" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L146" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L147" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K148" r:id="rId147"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9715,7 +9439,7 @@
       </c>
       <c r="B10" s="36" t="inlineStr">
         <is>
-          <t>O = KEYDIY/Xhorse 공용 폴딩 키날을 키웨이 상관없이 끼울 수 있음 (판매처 지정·안내 기준, 모델별 실측 자료는 없음). X = 전용 비상키/키날 포함/키날 없음/기판/판매처 미기재. 자세한 이유는 "공용 키날 비고" 칸 참고. 키날 목록은 Xhorse_키날_비상키_목록.xlsx</t>
+          <t>O = KEYDIY/Xhorse 공용 폴딩 키날을 키웨이 상관없이 끼울 수 있음 (판매처 지정·안내 기준, 모델별 실측 자료는 없음). X = 전용 비상키/키날 포함/키날 없음/기판/판매처 미기재. X인 이유는 마지막 "비고" 칸 참고. 키날 목록은 Xhorse_키날_비상키_목록.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite blade remark column in plain language with evidence; move it to last column
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -610,7 +610,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -671,7 +671,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>비고 (공용 키날 X 사유)</t>
+          <t>비고 (공용 키날 X 이유 / 추가 근거)</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>차고문 리모컨</t>
+          <t>차고문·게이트용 리모컨이에요. 자동차 키가 아니라서 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Garage Style … Remote Control"</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>키날 포함 제품 (TOY43 고정)</t>
+          <t>리모컨 머리에 토요타용 키날(TOY43 규격)이 처음부터 붙어서 나오는 제품이에요. 키날을 빼고 다른 키날로 바꿔 끼우는 구조가 아니라서 공용 키날을 쓰지 않아요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 상품명 "Key Head Remote … TOY43"</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>키날 포함 제품 (TOY43 고정)</t>
+          <t>리모컨 머리에 토요타용 키날(TOY43 규격)이 처음부터 붙어서 나오는 제품이에요. 키날을 빼고 다른 키날로 바꿔 끼우는 구조가 아니라서 공용 키날을 쓰지 않아요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 상품명 "Key Head Remote … TOY43"</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>키날 포함 제품 (TOY43 고정)</t>
+          <t>리모컨 머리에 토요타용 키날(TOY43 규격)이 처음부터 붙어서 나오는 제품이에요. 키날을 빼고 다른 키날로 바꿔 끼우는 구조가 아니라서 공용 키날을 쓰지 않아요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 상품명 "Key Head Remote … TOY43"</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>차고문 리모컨</t>
+          <t>차고문·게이트용 리모컨이에요. 자동차 키가 아니라서 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Garage Style … Remote Control"</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3455,7 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="L51" s="5" t="inlineStr">
         <is>
-          <t>키날 포함 제품 (TOY43 고정)</t>
+          <t>리모컨 머리에 토요타용 키날(TOY43 규격)이 처음부터 붙어서 나오는 제품이에요. 키날을 빼고 다른 키날로 바꿔 끼우는 구조가 아니라서 공용 키날을 쓰지 않아요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 상품명 "Key Head Remote … TOY43"</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
-          <t>키날 포함 제품 (TOY43 고정)</t>
+          <t>리모컨 머리에 토요타용 키날(TOY43 규격)이 처음부터 붙어서 나오는 제품이에요. 키날을 빼고 다른 키날로 바꿔 끼우는 구조가 아니라서 공용 키날을 쓰지 않아요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 상품명 "Key Head Remote … TOY43"</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="L55" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="L56" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3855,7 +3855,7 @@
       </c>
       <c r="L57" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="L58" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="L59" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="L60" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4207,7 @@
       </c>
       <c r="L63" s="12" t="inlineStr">
         <is>
-          <t>키날 없는 리모컨 단독형 (판매처 키날 항목 없음)</t>
+          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5107,7 @@
       </c>
       <c r="L79" s="25" t="inlineStr">
         <is>
-          <t>키날 포함 제품</t>
+          <t>비상키가 들어 있는 제품이라 키날을 따로 살 필요가 없어요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 키 규격 BW9MH (BMW 오토바이)</t>
         </is>
       </c>
     </row>
@@ -5167,7 +5167,7 @@
       </c>
       <c r="L80" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="L81" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="L82" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="L83" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="L84" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="L85" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5527,7 @@
       </c>
       <c r="L86" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -5699,7 +5699,7 @@
       </c>
       <c r="L89" s="25" t="inlineStr">
         <is>
-          <t>아우디·포르쉐 HU162 전용 비상키</t>
+          <t>아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
         </is>
       </c>
     </row>
@@ -5759,7 +5759,7 @@
       </c>
       <c r="L90" s="25" t="inlineStr">
         <is>
-          <t>아우디·포르쉐 HU162 전용 비상키</t>
+          <t>아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="L91" s="25" t="inlineStr">
         <is>
-          <t>아우디·포르쉐 HU162 전용 비상키</t>
+          <t>아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
         </is>
       </c>
     </row>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="L92" s="25" t="inlineStr">
         <is>
-          <t>아우디·포르쉐 HU162 전용 비상키</t>
+          <t>아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
         </is>
       </c>
     </row>
@@ -6163,7 +6163,7 @@
       </c>
       <c r="L97" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6223,7 @@
       </c>
       <c r="L98" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -6283,7 +6283,7 @@
       </c>
       <c r="L99" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -6343,7 +6343,7 @@
       </c>
       <c r="L100" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="L101" s="25" t="inlineStr">
         <is>
-          <t>UHS: 기판만 판매(Board only), 비상키 미포함. 아우디 A4·A5·A6·A7·A8·Q5 (2008~2016) 순정형 쉘에 넣는 기판 → 해당 쉘용 비상키 필요</t>
+          <t>아우디 순정 스마트키(2008~2016 A4·A5·A6·A7·A8·Q5) 케이스에 넣는 기판만 파는 제품이에요. 비상키는 그 아우디 케이스에 맞는 것을 써야 해요. [근거] UHS: "Board only(기판만)", "Emergency Blade (not included)", 적용 차종 목록</t>
         </is>
       </c>
     </row>
@@ -6463,7 +6463,7 @@
       </c>
       <c r="L102" s="25" t="inlineStr">
         <is>
-          <t>기판만 판매. 쉘에 맞는 비상키 필요</t>
+          <t>BMW 스마트키용 기판만 파는 제품이에요(쉘·키날·배터리 없음). 비상키는 기판을 넣을 BMW 쉘에 맞는 것을 따로 준비해야 해요. [근거] ABKEYS: "PCB board only, No shell included, Key blade is not included"</t>
         </is>
       </c>
     </row>
@@ -6523,7 +6523,7 @@
       </c>
       <c r="L103" s="25" t="inlineStr">
         <is>
-          <t>기판만 판매. 쉘에 맞는 비상키 필요</t>
+          <t>BMW 스마트키용 기판만 파는 제품이에요(쉘·키날·배터리 없음). 비상키는 기판을 넣을 BMW 쉘에 맞는 것을 따로 준비해야 해요. [근거] ABKEYS: "PCB board only, No shell included, Key blade is not included"</t>
         </is>
       </c>
     </row>
@@ -6637,7 +6637,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L105" s="25" t="n"/>
+      <c r="L105" s="25" t="inlineStr">
+        <is>
+          <t>[추가 근거] key4: "키날 미포함, 공용 폴딩 키날(universal flip remote key blades)을 구매하라"고 안내</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="22" t="inlineStr">
@@ -6749,7 +6753,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L107" s="25" t="n"/>
+      <c r="L107" s="25" t="inlineStr">
+        <is>
+          <t>[추가 근거] 나이프(접히는 칼) 모양 스마트키. UHS·Locksmith Keyless: "Blade NOT included(키날 미포함)", 키날은 따로 사서 끼움</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="22" t="inlineStr">
@@ -6915,7 +6923,7 @@
       </c>
       <c r="L110" s="25" t="inlineStr">
         <is>
-          <t>키날 없는 제품</t>
+          <t>카드 모양 스마트키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS: "The Xhorse card key doesn't have a key blade"</t>
         </is>
       </c>
     </row>
@@ -6971,7 +6979,7 @@
       </c>
       <c r="L111" s="25" t="inlineStr">
         <is>
-          <t>키날 없는 제품</t>
+          <t>카드 모양 스마트키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS: "The Xhorse card key doesn't have a key blade"</t>
         </is>
       </c>
     </row>
@@ -7197,7 +7205,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L115" s="25" t="n"/>
+      <c r="L115" s="25" t="inlineStr">
+        <is>
+          <t>[추가 근거] 같은 모양의 3버튼 버전(XSKFF1EN)에 ABKEYS가 공용 폴딩 키날을 맞는 부품으로 지정. Best Key Supply: 키날 미포함, "원하는 키날을 끼워 조립" 안내</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="22" t="inlineStr">
@@ -7255,7 +7267,7 @@
       </c>
       <c r="L116" s="25" t="inlineStr">
         <is>
-          <t>닛산 NSN14 전용 비상키</t>
+          <t>닛산 스마트키 모양이라 닛산 스마트키용 비상키(NSN14 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Nissan 2007-2025 Smart Key Blade H0564-EG010, NSN14"를 지정</t>
         </is>
       </c>
     </row>
@@ -7427,7 +7439,7 @@
       </c>
       <c r="L119" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -7487,7 +7499,7 @@
       </c>
       <c r="L120" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7559,7 @@
       </c>
       <c r="L121" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7619,7 @@
       </c>
       <c r="L122" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -7667,7 +7679,7 @@
       </c>
       <c r="L123" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -7727,7 +7739,7 @@
       </c>
       <c r="L124" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -7787,7 +7799,7 @@
       </c>
       <c r="L125" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 TOY48 전용 비상키</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -7847,7 +7859,7 @@
       </c>
       <c r="L126" s="25" t="inlineStr">
         <is>
-          <t>판매처 간 상충: key4는 공용 폴딩 키날 안내, 같은 XM38 토요타형(XSTO01EN)은 ABKEYS가 TOY48 전용 비상키 지정 → 구매 전 확인 필요</t>
+          <t>판매처마다 말이 달라 확인이 필요해요. [근거] key4는 "공용 폴딩 키날을 구매하라"고 안내. 반면 같은 XM38 토요타 모양(XSTO01EN)은 ABKEYS가 토요타 스마트키용 비상키(TOY48)를 지정. 모양이 토요타 스마트키형이라 TOY48 비상키일 가능성이 높음</t>
         </is>
       </c>
     </row>
@@ -7963,7 +7975,7 @@
       </c>
       <c r="L128" s="25" t="inlineStr">
         <is>
-          <t>키날 포함 제품</t>
+          <t>비상키가 들어 있는 제품이라 키날을 따로 살 필요가 없어요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 키 규격 CY22. 단 같은 페이지 안내문에는 "키날 미포함"이라는 문구도 있어 판매처에 확인 권장</t>
         </is>
       </c>
     </row>
@@ -8023,7 +8035,7 @@
       </c>
       <c r="L129" s="25" t="inlineStr">
         <is>
-          <t>ABKEYS가 랜드로버 HU101 전용 스마트키 비상키 지정 (key4는 공용 폴딩 키날 안내 → 판매처 간 상충)</t>
+          <t>랜드로버 스마트키 모양이라 랜드로버 스마트키용 비상키(HU101 규격)를 끼우는 것으로 보여요. [근거] ABKEYS가 "Range Rover, Land Rover 2010+ Smart Key Blade, HU101"을 지정, 3D Group도 "Blade Reference HU101". 단 key4는 공용 폴딩 키날 구매를 안내해서 판매처마다 말이 달라요 → 구매 전 확인 필요</t>
         </is>
       </c>
     </row>
@@ -8083,7 +8095,7 @@
       </c>
       <c r="L130" s="25" t="inlineStr">
         <is>
-          <t>Locksmith Keyless 등 다른 판매처도 키날 정보 없음. 같은 랜드로버형 XSLR01EN은 HU101 전용 비상키 지정 → 확인 필요</t>
+          <t>키날 정보를 적은 판매처를 찾지 못했어요. [근거] Locksmith Keyless 등 설명에 키날 언급 없음. 같은 랜드로버 모양(XSLR01EN)은 ABKEYS가 랜드로버 스마트키용 비상키(HU101)를 지정 → 같은 방식일 가능성이 높지만 확인 필요</t>
         </is>
       </c>
     </row>
@@ -8139,7 +8151,7 @@
       </c>
       <c r="L131" s="25" t="inlineStr">
         <is>
-          <t>키날 없는 제품</t>
+          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
         </is>
       </c>
     </row>
@@ -8195,7 +8207,7 @@
       </c>
       <c r="L132" s="25" t="inlineStr">
         <is>
-          <t>키날 없는 제품</t>
+          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8263,7 @@
       </c>
       <c r="L133" s="25" t="inlineStr">
         <is>
-          <t>키날 없는 제품</t>
+          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
         </is>
       </c>
     </row>
@@ -8311,7 +8323,7 @@
       </c>
       <c r="L134" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8371,7 +8383,7 @@
       </c>
       <c r="L135" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>아우디·폭스바겐 MQB48 폴딩키용 기판만 파는 제품이에요(케이스 없음). 키날은 기판을 넣을 폴딩키 케이스에 맞는 것을 따로 준비해야 해요. [근거] ABKEYS: "PCB board only, key cover not included". 맞는 키날 정보는 판매처에 없음</t>
         </is>
       </c>
     </row>
@@ -8431,7 +8443,7 @@
       </c>
       <c r="L136" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8491,7 +8503,7 @@
       </c>
       <c r="L137" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8551,7 +8563,7 @@
       </c>
       <c r="L138" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8611,7 +8623,7 @@
       </c>
       <c r="L139" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8671,7 +8683,7 @@
       </c>
       <c r="L140" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8731,7 +8743,7 @@
       </c>
       <c r="L141" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8791,7 +8803,7 @@
       </c>
       <c r="L142" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8851,7 +8863,7 @@
       </c>
       <c r="L143" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>아우디·폭스바겐 MQB48 폴딩키용 기판만 파는 제품이에요(케이스 없음). 키날은 기판을 넣을 폴딩키 케이스에 맞는 것을 따로 준비해야 해요. [근거] ABKEYS: "PCB board only, key cover not included". 맞는 키날 정보는 판매처에 없음</t>
         </is>
       </c>
     </row>
@@ -8911,7 +8923,7 @@
       </c>
       <c r="L144" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -8971,7 +8983,7 @@
       </c>
       <c r="L145" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -9031,7 +9043,7 @@
       </c>
       <c r="L146" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -9091,7 +9103,7 @@
       </c>
       <c r="L147" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>
@@ -9151,7 +9163,7 @@
       </c>
       <c r="L148" s="32" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 키날 필요</t>
+          <t>특정 브랜드 스마트키 케이스에 넣는 기판만 파는 제품이에요(케이스·비상키 없음). 비상키는 기판을 넣을 케이스에 맞는 것을 따로 준비해야 해요. [근거] 판매처 상품명·설명 "Special PCB Board", "Without Key Shell"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep remarks only for X rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>비고 (공용 키날 X 이유 / 추가 근거)</t>
+          <t>비고 (공용 키날 X 이유)</t>
         </is>
       </c>
     </row>
@@ -6637,11 +6637,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L105" s="25" t="inlineStr">
-        <is>
-          <t>[추가 근거] key4: "키날 미포함, 공용 폴딩 키날(universal flip remote key blades)을 구매하라"고 안내</t>
-        </is>
-      </c>
+      <c r="L105" s="25" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="22" t="inlineStr">
@@ -6753,11 +6749,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L107" s="25" t="inlineStr">
-        <is>
-          <t>[추가 근거] 나이프(접히는 칼) 모양 스마트키. UHS·Locksmith Keyless: "Blade NOT included(키날 미포함)", 키날은 따로 사서 끼움</t>
-        </is>
-      </c>
+      <c r="L107" s="25" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="22" t="inlineStr">
@@ -7205,11 +7197,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L115" s="25" t="inlineStr">
-        <is>
-          <t>[추가 근거] 같은 모양의 3버튼 버전(XSKFF1EN)에 ABKEYS가 공용 폴딩 키날을 맞는 부품으로 지정. Best Key Supply: 키날 미포함, "원하는 키날을 끼워 조립" 안내</t>
-        </is>
-      </c>
+      <c r="L115" s="25" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Move XS PCB-only models to bottom of XS section with remark
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -5656,40 +5656,40 @@
       </c>
       <c r="C89" s="22" t="inlineStr">
         <is>
-          <t>XSMA41EN</t>
+          <t>XSMQB1EN</t>
         </is>
       </c>
       <c r="D89" s="22" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>MQB</t>
         </is>
       </c>
       <c r="E89" s="22" t="inlineStr">
         <is>
-          <t>스마트키 기판</t>
-        </is>
-      </c>
-      <c r="F89" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+          <t>스마트키</t>
+        </is>
+      </c>
+      <c r="F89" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G89" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H89" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I89" s="26" t="n">
-        <v>34.99</v>
+        <v>19.99</v>
       </c>
       <c r="J89" s="25" t="inlineStr">
         <is>
-          <t>Xhorse XSMA41EN Smart Key Board With 3Buttons for Audi MLB Cars</t>
+          <t>Xhorse Universal Smart Key XSMQB1EN VW MQB Style 3Buttons</t>
         </is>
       </c>
       <c r="K89" s="27" t="inlineStr">
@@ -5697,11 +5697,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L89" s="25" t="inlineStr">
-        <is>
-          <t>아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
-        </is>
-      </c>
+      <c r="L89" s="25" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="22" t="inlineStr">
@@ -5716,40 +5712,40 @@
       </c>
       <c r="C90" s="22" t="inlineStr">
         <is>
-          <t>XSMA4YEN</t>
+          <t>XSSC01EN</t>
         </is>
       </c>
       <c r="D90" s="22" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>Supercar</t>
         </is>
       </c>
       <c r="E90" s="22" t="inlineStr">
         <is>
-          <t>스마트키 기판</t>
-        </is>
-      </c>
-      <c r="F90" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+          <t>스마트키</t>
+        </is>
+      </c>
+      <c r="F90" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G90" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H90" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I90" s="26" t="n">
-        <v>38.99</v>
+        <v>32</v>
       </c>
       <c r="J90" s="25" t="inlineStr">
         <is>
-          <t>Xhorse XSMA4YEN Smart Key Board With 3Buttons for Audi A4 MLB Cars Works with Xhorse MLB Tool</t>
+          <t>Xhorse Universal Smart Key XSSC01EN Supercar Style Marble Black Color XM38 3Buttons</t>
         </is>
       </c>
       <c r="K90" s="27" t="inlineStr">
@@ -5757,11 +5753,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L90" s="25" t="inlineStr">
-        <is>
-          <t>아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
-        </is>
-      </c>
+      <c r="L90" s="25" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="22" t="inlineStr">
@@ -5776,40 +5768,40 @@
       </c>
       <c r="C91" s="22" t="inlineStr">
         <is>
-          <t>XSMA8YEN</t>
+          <t>XSSC04EN</t>
         </is>
       </c>
       <c r="D91" s="22" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>Supercar</t>
         </is>
       </c>
       <c r="E91" s="22" t="inlineStr">
         <is>
-          <t>스마트키 기판</t>
-        </is>
-      </c>
-      <c r="F91" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+          <t>스마트키</t>
+        </is>
+      </c>
+      <c r="F91" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G91" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H91" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I91" s="26" t="n">
-        <v>38.99</v>
+        <v>32</v>
       </c>
       <c r="J91" s="25" t="inlineStr">
         <is>
-          <t>Xhorse XSMA8YEN Smart Key Board With 3Buttons for Audi A8 MLB Cars Works with Xhorse MLB Tool</t>
+          <t>Xhorse Universal Smart Key XSSC04EN Supercar Style Miami Blue Color XM38 3Buttons</t>
         </is>
       </c>
       <c r="K91" s="27" t="inlineStr">
@@ -5817,11 +5809,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L91" s="25" t="inlineStr">
-        <is>
-          <t>아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
-        </is>
-      </c>
+      <c r="L91" s="25" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="22" t="inlineStr">
@@ -5836,40 +5824,40 @@
       </c>
       <c r="C92" s="22" t="inlineStr">
         <is>
-          <t>XSMPSYEN</t>
+          <t>XSSC05EN</t>
         </is>
       </c>
       <c r="D92" s="22" t="inlineStr">
         <is>
-          <t>Porsche</t>
+          <t>Supercar</t>
         </is>
       </c>
       <c r="E92" s="22" t="inlineStr">
         <is>
-          <t>스마트키 기판</t>
-        </is>
-      </c>
-      <c r="F92" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+          <t>스마트키</t>
+        </is>
+      </c>
+      <c r="F92" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G92" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H92" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I92" s="26" t="n">
-        <v>38.99</v>
+        <v>32</v>
       </c>
       <c r="J92" s="25" t="inlineStr">
         <is>
-          <t>Xhorse XSMPSYEN Smart Key Board With 3Buttons for Porsche MLB Cars Works with Xhorse MLB Tool</t>
+          <t>Xhorse Universal Smart Key XSSC05EN Supercar Style Marble Grey Color XM38 3Buttons</t>
         </is>
       </c>
       <c r="K92" s="27" t="inlineStr">
@@ -5877,11 +5865,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L92" s="25" t="inlineStr">
-        <is>
-          <t>아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
-        </is>
-      </c>
+      <c r="L92" s="25" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="22" t="inlineStr">
@@ -5896,12 +5880,12 @@
       </c>
       <c r="C93" s="22" t="inlineStr">
         <is>
-          <t>XSMQB1EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D93" s="22" t="inlineStr">
         <is>
-          <t>MQB</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E93" s="22" t="inlineStr">
@@ -5909,27 +5893,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F93" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F93" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G93" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H93" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I93" s="26" t="n">
-        <v>19.99</v>
+        <v>47</v>
       </c>
       <c r="J93" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSMQB1EN VW MQB Style 3Buttons</t>
+          <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K93" s="27" t="inlineStr">
@@ -5937,7 +5921,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L93" s="25" t="n"/>
+      <c r="L93" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="22" t="inlineStr">
@@ -5952,12 +5940,12 @@
       </c>
       <c r="C94" s="22" t="inlineStr">
         <is>
-          <t>XSSC01EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D94" s="22" t="inlineStr">
         <is>
-          <t>Supercar</t>
+          <t>Lexus</t>
         </is>
       </c>
       <c r="E94" s="22" t="inlineStr">
@@ -5965,27 +5953,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F94" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F94" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G94" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H94" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I94" s="26" t="n">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="J94" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSSC01EN Supercar Style Marble Black Color XM38 3Buttons</t>
+          <t>Xhorse Lexus Smart Key 315/433MHz 3Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K94" s="27" t="inlineStr">
@@ -5993,7 +5981,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L94" s="25" t="n"/>
+      <c r="L94" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="22" t="inlineStr">
@@ -6008,12 +6000,12 @@
       </c>
       <c r="C95" s="22" t="inlineStr">
         <is>
-          <t>XSSC04EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D95" s="22" t="inlineStr">
         <is>
-          <t>Supercar</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E95" s="22" t="inlineStr">
@@ -6021,27 +6013,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F95" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F95" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G95" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H95" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I95" s="26" t="n">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="J95" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSSC04EN Supercar Style Miami Blue Color XM38 3Buttons</t>
+          <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K95" s="27" t="inlineStr">
@@ -6049,7 +6041,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L95" s="25" t="n"/>
+      <c r="L95" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="22" t="inlineStr">
@@ -6064,12 +6060,12 @@
       </c>
       <c r="C96" s="22" t="inlineStr">
         <is>
-          <t>XSSC05EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D96" s="22" t="inlineStr">
         <is>
-          <t>Supercar</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E96" s="22" t="inlineStr">
@@ -6077,27 +6073,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F96" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F96" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G96" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H96" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I96" s="26" t="n">
-        <v>32</v>
+        <v>49.99</v>
       </c>
       <c r="J96" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSSC05EN Supercar Style Marble Grey Color XM38 3Buttons</t>
+          <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K96" s="27" t="inlineStr">
@@ -6105,7 +6101,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L96" s="25" t="n"/>
+      <c r="L96" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="22" t="inlineStr">
@@ -6115,17 +6115,17 @@
       </c>
       <c r="B97" s="23" t="inlineStr">
         <is>
-          <t>3버튼</t>
+          <t>4버튼</t>
         </is>
       </c>
       <c r="C97" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSCH01EN</t>
         </is>
       </c>
       <c r="D97" s="22" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Chrysler</t>
         </is>
       </c>
       <c r="E97" s="22" t="inlineStr">
@@ -6133,27 +6133,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F97" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F97" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G97" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H97" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I97" s="26" t="n">
-        <v>47</v>
+        <v>18.5</v>
       </c>
       <c r="J97" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSCH01EN Chrysler Style XM38 4Buttons</t>
         </is>
       </c>
       <c r="K97" s="27" t="inlineStr">
@@ -6161,11 +6161,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L97" s="25" t="inlineStr">
-        <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
-        </is>
-      </c>
+      <c r="L97" s="25" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="22" t="inlineStr">
@@ -6175,17 +6171,17 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>3버튼</t>
+          <t>4버튼</t>
         </is>
       </c>
       <c r="C98" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSCL01EN</t>
         </is>
       </c>
       <c r="D98" s="22" t="inlineStr">
         <is>
-          <t>Lexus</t>
+          <t>Chevrolet</t>
         </is>
       </c>
       <c r="E98" s="22" t="inlineStr">
@@ -6193,27 +6189,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F98" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F98" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G98" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H98" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I98" s="26" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="J98" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Lexus Smart Key 315/433MHz 3Buttons XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSCL01EN Chevrolet Style 4Buttons</t>
         </is>
       </c>
       <c r="K98" s="27" t="inlineStr">
@@ -6221,11 +6217,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L98" s="25" t="inlineStr">
-        <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
-        </is>
-      </c>
+      <c r="L98" s="25" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="22" t="inlineStr">
@@ -6235,17 +6227,17 @@
       </c>
       <c r="B99" s="23" t="inlineStr">
         <is>
-          <t>3버튼</t>
+          <t>4버튼</t>
         </is>
       </c>
       <c r="C99" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSCS00EN</t>
         </is>
       </c>
       <c r="D99" s="22" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Hyundai</t>
         </is>
       </c>
       <c r="E99" s="22" t="inlineStr">
@@ -6253,27 +6245,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F99" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F99" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G99" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H99" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I99" s="26" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="J99" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSCS00EN Hyundai Style 4Buttons</t>
         </is>
       </c>
       <c r="K99" s="27" t="inlineStr">
@@ -6281,11 +6273,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L99" s="25" t="inlineStr">
-        <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
-        </is>
-      </c>
+      <c r="L99" s="25" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="22" t="inlineStr">
@@ -6295,17 +6283,17 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>3버튼</t>
+          <t>4버튼</t>
         </is>
       </c>
       <c r="C100" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSDFX2EN</t>
         </is>
       </c>
       <c r="D100" s="22" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Knife</t>
         </is>
       </c>
       <c r="E100" s="22" t="inlineStr">
@@ -6313,27 +6301,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F100" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F100" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G100" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H100" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I100" s="26" t="n">
-        <v>49.99</v>
+        <v>18</v>
       </c>
       <c r="J100" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Toyota Smart Key 315/433MHz 3Buttons XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSDFX2EN Knife Style 4Buttons</t>
         </is>
       </c>
       <c r="K100" s="27" t="inlineStr">
@@ -6341,11 +6329,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L100" s="25" t="inlineStr">
-        <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
-        </is>
-      </c>
+      <c r="L100" s="25" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="22" t="inlineStr">
@@ -6360,12 +6344,12 @@
       </c>
       <c r="C101" s="22" t="inlineStr">
         <is>
-          <t>XSADJ1EN</t>
+          <t>XSFO02EN</t>
         </is>
       </c>
       <c r="D101" s="22" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>Ford</t>
         </is>
       </c>
       <c r="E101" s="22" t="inlineStr">
@@ -6373,27 +6357,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F101" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F101" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G101" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H101" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I101" s="26" t="n">
-        <v>44.99</v>
+        <v>18.5</v>
       </c>
       <c r="J101" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key For Audi 315MHz 433MHz 868MHz 4Buttons XSADJ1EN</t>
+          <t>Xhorse Universal Smart Key XSFO02EN Ford Style XM38 4Buttons</t>
         </is>
       </c>
       <c r="K101" s="27" t="inlineStr">
@@ -6401,11 +6385,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L101" s="25" t="inlineStr">
-        <is>
-          <t>아우디 순정 스마트키(2008~2016 A4·A5·A6·A7·A8·Q5) 케이스에 넣는 기판만 파는 제품이에요. 비상키는 그 아우디 케이스에 맞는 것을 써야 해요. [근거] UHS: "Board only(기판만)", "Emergency Blade (not included)", 적용 차종 목록</t>
-        </is>
-      </c>
+      <c r="L101" s="25" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="22" t="inlineStr">
@@ -6420,40 +6400,40 @@
       </c>
       <c r="C102" s="22" t="inlineStr">
         <is>
-          <t>XSBMB1EN</t>
+          <t>XSGA80EN</t>
         </is>
       </c>
       <c r="D102" s="22" t="inlineStr">
         <is>
-          <t>Bread</t>
+          <t>VW</t>
         </is>
       </c>
       <c r="E102" s="22" t="inlineStr">
         <is>
-          <t>스마트키 기판</t>
-        </is>
-      </c>
-      <c r="F102" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+          <t>스마트키</t>
+        </is>
+      </c>
+      <c r="F102" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G102" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H102" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I102" s="26" t="n">
-        <v>19.99</v>
+        <v>19</v>
       </c>
       <c r="J102" s="25" t="inlineStr">
         <is>
-          <t>Xhorse XSBMB1EN BMW Smart Key PCB BMW Bread Style for F/G Chassis BDC2 BDC3 4Buttons</t>
+          <t>Xhorse Universal Smart Key XSGA80EN VW Style XM38 4Buttons</t>
         </is>
       </c>
       <c r="K102" s="27" t="inlineStr">
@@ -6461,11 +6441,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L102" s="25" t="inlineStr">
-        <is>
-          <t>BMW 스마트키용 기판만 파는 제품이에요(쉘·키날·배터리 없음). 비상키는 기판을 넣을 BMW 쉘에 맞는 것을 따로 준비해야 해요. [근거] ABKEYS: "PCB board only, No shell included, Key blade is not included"</t>
-        </is>
-      </c>
+      <c r="L102" s="25" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="22" t="inlineStr">
@@ -6480,17 +6456,13 @@
       </c>
       <c r="C103" s="22" t="inlineStr">
         <is>
-          <t>XSBMU1EN</t>
-        </is>
-      </c>
-      <c r="D103" s="22" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
+          <t>XSKC04EN</t>
+        </is>
+      </c>
+      <c r="D103" s="22" t="inlineStr"/>
       <c r="E103" s="22" t="inlineStr">
         <is>
-          <t>스마트키 기판</t>
+          <t>스마트키</t>
         </is>
       </c>
       <c r="F103" s="24" t="inlineStr">
@@ -6500,20 +6472,20 @@
       </c>
       <c r="G103" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H103" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I103" s="26" t="n">
-        <v>19.99</v>
+        <v>29.99</v>
       </c>
       <c r="J103" s="25" t="inlineStr">
         <is>
-          <t>Xhorse XSBMU1EN BMW Smart Key PCB BMW U Style for F/G Chassis BDC2 BDC3 4Buttons</t>
+          <t>Xhorse King Card Slimmest Universal Smart Key 4Buttons XSKC04EN Diamond Blue Colour</t>
         </is>
       </c>
       <c r="K103" s="27" t="inlineStr">
@@ -6523,7 +6495,7 @@
       </c>
       <c r="L103" s="25" t="inlineStr">
         <is>
-          <t>BMW 스마트키용 기판만 파는 제품이에요(쉘·키날·배터리 없음). 비상키는 기판을 넣을 BMW 쉘에 맞는 것을 따로 준비해야 해요. [근거] ABKEYS: "PCB board only, No shell included, Key blade is not included"</t>
+          <t>카드 모양 스마트키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS: "The Xhorse card key doesn't have a key blade"</t>
         </is>
       </c>
     </row>
@@ -6540,40 +6512,36 @@
       </c>
       <c r="C104" s="22" t="inlineStr">
         <is>
-          <t>XSCH01EN</t>
-        </is>
-      </c>
-      <c r="D104" s="22" t="inlineStr">
-        <is>
-          <t>Chrysler</t>
-        </is>
-      </c>
+          <t>XSKC05EN</t>
+        </is>
+      </c>
+      <c r="D104" s="22" t="inlineStr"/>
       <c r="E104" s="22" t="inlineStr">
         <is>
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F104" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F104" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G104" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H104" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I104" s="26" t="n">
-        <v>18.5</v>
+        <v>29.99</v>
       </c>
       <c r="J104" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSCH01EN Chrysler Style XM38 4Buttons</t>
+          <t>Xhorse King Card Slimmest Universal Smart Key 4Buttons XSKC05EN Sky Blue Colour</t>
         </is>
       </c>
       <c r="K104" s="27" t="inlineStr">
@@ -6581,7 +6549,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L104" s="25" t="n"/>
+      <c r="L104" s="25" t="inlineStr">
+        <is>
+          <t>카드 모양 스마트키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS: "The Xhorse card key doesn't have a key blade"</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="22" t="inlineStr">
@@ -6596,12 +6568,12 @@
       </c>
       <c r="C105" s="22" t="inlineStr">
         <is>
-          <t>XSCL01EN</t>
+          <t>XSKF20EN</t>
         </is>
       </c>
       <c r="D105" s="22" t="inlineStr">
         <is>
-          <t>Chevrolet</t>
+          <t>BMW</t>
         </is>
       </c>
       <c r="E105" s="22" t="inlineStr">
@@ -6625,11 +6597,11 @@
         </is>
       </c>
       <c r="I105" s="26" t="n">
-        <v>18</v>
+        <v>18.59</v>
       </c>
       <c r="J105" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSCL01EN Chevrolet Style 4Buttons</t>
+          <t>Xhorse Universal Smart Key XSKF20EN BMW Style 4Buttons</t>
         </is>
       </c>
       <c r="K105" s="27" t="inlineStr">
@@ -6652,12 +6624,12 @@
       </c>
       <c r="C106" s="22" t="inlineStr">
         <is>
-          <t>XSCS00EN</t>
+          <t>XSKF21EN</t>
         </is>
       </c>
       <c r="D106" s="22" t="inlineStr">
         <is>
-          <t>Hyundai</t>
+          <t>BMW</t>
         </is>
       </c>
       <c r="E106" s="22" t="inlineStr">
@@ -6681,11 +6653,11 @@
         </is>
       </c>
       <c r="I106" s="26" t="n">
-        <v>18</v>
+        <v>18.59</v>
       </c>
       <c r="J106" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSCS00EN Hyundai Style 4Buttons</t>
+          <t>Xhorse Universal Smart Key XSKF21EN BMW Style 4Buttons</t>
         </is>
       </c>
       <c r="K106" s="27" t="inlineStr">
@@ -6708,7 +6680,7 @@
       </c>
       <c r="C107" s="22" t="inlineStr">
         <is>
-          <t>XSDFX2EN</t>
+          <t>XSKF30EN</t>
         </is>
       </c>
       <c r="D107" s="22" t="inlineStr">
@@ -6737,11 +6709,11 @@
         </is>
       </c>
       <c r="I107" s="26" t="n">
-        <v>18</v>
+        <v>18.59</v>
       </c>
       <c r="J107" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSDFX2EN Knife Style 4Buttons</t>
+          <t>Xhorse Universal Smart Key XSKF30EN Knife Style 4Buttons</t>
         </is>
       </c>
       <c r="K107" s="27" t="inlineStr">
@@ -6764,12 +6736,12 @@
       </c>
       <c r="C108" s="22" t="inlineStr">
         <is>
-          <t>XSFO02EN</t>
+          <t>XSKFF0EN</t>
         </is>
       </c>
       <c r="D108" s="22" t="inlineStr">
         <is>
-          <t>Ford</t>
+          <t>Knife</t>
         </is>
       </c>
       <c r="E108" s="22" t="inlineStr">
@@ -6784,20 +6756,20 @@
       </c>
       <c r="G108" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H108" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I108" s="26" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
       <c r="J108" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSFO02EN Ford Style XM38 4Buttons</t>
+          <t>Xhorse Universal Smart Key XSKFF0EN Knife Style 4Buttons</t>
         </is>
       </c>
       <c r="K108" s="27" t="inlineStr">
@@ -6820,12 +6792,12 @@
       </c>
       <c r="C109" s="22" t="inlineStr">
         <is>
-          <t>XSGA80EN</t>
+          <t>XSNIS2EN</t>
         </is>
       </c>
       <c r="D109" s="22" t="inlineStr">
         <is>
-          <t>VW</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="E109" s="22" t="inlineStr">
@@ -6833,27 +6805,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F109" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F109" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G109" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H109" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I109" s="26" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="J109" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSGA80EN VW Style XM38 4Buttons</t>
+          <t>Xhorse Universal Smart Key XSNIS2EN Nissan Style 4Buttons</t>
         </is>
       </c>
       <c r="K109" s="27" t="inlineStr">
@@ -6861,7 +6833,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L109" s="25" t="n"/>
+      <c r="L109" s="25" t="inlineStr">
+        <is>
+          <t>닛산 스마트키 모양이라 닛산 스마트키용 비상키(NSN14 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Nissan 2007-2025 Smart Key Blade H0564-EG010, NSN14"를 지정</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="22" t="inlineStr">
@@ -6876,36 +6852,40 @@
       </c>
       <c r="C110" s="22" t="inlineStr">
         <is>
-          <t>XSKC04EN</t>
-        </is>
-      </c>
-      <c r="D110" s="22" t="inlineStr"/>
+          <t>XSPS01EN</t>
+        </is>
+      </c>
+      <c r="D110" s="22" t="inlineStr">
+        <is>
+          <t>Porsche</t>
+        </is>
+      </c>
       <c r="E110" s="22" t="inlineStr">
         <is>
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F110" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F110" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G110" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H110" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I110" s="26" t="n">
-        <v>29.99</v>
+        <v>18</v>
       </c>
       <c r="J110" s="25" t="inlineStr">
         <is>
-          <t>Xhorse King Card Slimmest Universal Smart Key 4Buttons XSKC04EN Diamond Blue Colour</t>
+          <t>Xhorse Universal Smart Key XSPS01EN Porsche Style XM38 4Buttons Red</t>
         </is>
       </c>
       <c r="K110" s="27" t="inlineStr">
@@ -6913,11 +6893,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L110" s="25" t="inlineStr">
-        <is>
-          <t>카드 모양 스마트키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS: "The Xhorse card key doesn't have a key blade"</t>
-        </is>
-      </c>
+      <c r="L110" s="25" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="22" t="inlineStr">
@@ -6932,36 +6908,40 @@
       </c>
       <c r="C111" s="22" t="inlineStr">
         <is>
-          <t>XSKC05EN</t>
-        </is>
-      </c>
-      <c r="D111" s="22" t="inlineStr"/>
+          <t>XSSBR0EN</t>
+        </is>
+      </c>
+      <c r="D111" s="22" t="inlineStr">
+        <is>
+          <t>Subaru</t>
+        </is>
+      </c>
       <c r="E111" s="22" t="inlineStr">
         <is>
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F111" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F111" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G111" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H111" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I111" s="26" t="n">
-        <v>29.99</v>
+        <v>18.5</v>
       </c>
       <c r="J111" s="25" t="inlineStr">
         <is>
-          <t>Xhorse King Card Slimmest Universal Smart Key 4Buttons XSKC05EN Sky Blue Colour</t>
+          <t>Xhorse Universal Smart Key XSSBR0EN Subaru Style XM38 4Buttons</t>
         </is>
       </c>
       <c r="K111" s="27" t="inlineStr">
@@ -6969,11 +6949,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L111" s="25" t="inlineStr">
-        <is>
-          <t>카드 모양 스마트키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS: "The Xhorse card key doesn't have a key blade"</t>
-        </is>
-      </c>
+      <c r="L111" s="25" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="22" t="inlineStr">
@@ -6988,12 +6964,12 @@
       </c>
       <c r="C112" s="22" t="inlineStr">
         <is>
-          <t>XSKF20EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D112" s="22" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E112" s="22" t="inlineStr">
@@ -7001,27 +6977,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F112" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F112" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G112" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H112" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I112" s="26" t="n">
-        <v>18.59</v>
+        <v>39.99</v>
       </c>
       <c r="J112" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSKF20EN BMW Style 4Buttons</t>
+          <t>Xhorse Toyota XM38 Smart Key 4Buttons Support 4D 8A 4A All in One With Key Shell XSTO01EN</t>
         </is>
       </c>
       <c r="K112" s="27" t="inlineStr">
@@ -7029,7 +7005,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L112" s="25" t="n"/>
+      <c r="L112" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="22" t="inlineStr">
@@ -7044,12 +7024,12 @@
       </c>
       <c r="C113" s="22" t="inlineStr">
         <is>
-          <t>XSKF21EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D113" s="22" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E113" s="22" t="inlineStr">
@@ -7057,27 +7037,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F113" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F113" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G113" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H113" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I113" s="26" t="n">
-        <v>18.59</v>
+        <v>47</v>
       </c>
       <c r="J113" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSKF21EN BMW Style 4Buttons</t>
+          <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons SUV XSTO01EN</t>
         </is>
       </c>
       <c r="K113" s="27" t="inlineStr">
@@ -7085,7 +7065,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L113" s="25" t="n"/>
+      <c r="L113" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="22" t="inlineStr">
@@ -7100,12 +7084,12 @@
       </c>
       <c r="C114" s="22" t="inlineStr">
         <is>
-          <t>XSKF30EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D114" s="22" t="inlineStr">
         <is>
-          <t>Knife</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E114" s="22" t="inlineStr">
@@ -7113,27 +7097,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F114" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F114" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G114" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H114" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I114" s="26" t="n">
-        <v>18.59</v>
+        <v>47</v>
       </c>
       <c r="J114" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSKF30EN Knife Style 4Buttons</t>
+          <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K114" s="27" t="inlineStr">
@@ -7141,7 +7125,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L114" s="25" t="n"/>
+      <c r="L114" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="22" t="inlineStr">
@@ -7156,12 +7144,12 @@
       </c>
       <c r="C115" s="22" t="inlineStr">
         <is>
-          <t>XSKFF0EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D115" s="22" t="inlineStr">
         <is>
-          <t>Knife</t>
+          <t>Lexus</t>
         </is>
       </c>
       <c r="E115" s="22" t="inlineStr">
@@ -7169,27 +7157,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F115" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F115" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G115" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H115" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I115" s="26" t="n">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="J115" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSKFF0EN Knife Style 4Buttons</t>
+          <t>Xhorse Lexus Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K115" s="27" t="inlineStr">
@@ -7197,7 +7185,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L115" s="25" t="n"/>
+      <c r="L115" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="22" t="inlineStr">
@@ -7212,12 +7204,12 @@
       </c>
       <c r="C116" s="22" t="inlineStr">
         <is>
-          <t>XSNIS2EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D116" s="22" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E116" s="22" t="inlineStr">
@@ -7232,20 +7224,20 @@
       </c>
       <c r="G116" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H116" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I116" s="26" t="n">
-        <v>18.5</v>
+        <v>49</v>
       </c>
       <c r="J116" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSNIS2EN Nissan Style 4Buttons</t>
+          <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K116" s="27" t="inlineStr">
@@ -7255,7 +7247,7 @@
       </c>
       <c r="L116" s="25" t="inlineStr">
         <is>
-          <t>닛산 스마트키 모양이라 닛산 스마트키용 비상키(NSN14 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Nissan 2007-2025 Smart Key Blade H0564-EG010, NSN14"를 지정</t>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
         </is>
       </c>
     </row>
@@ -7272,12 +7264,12 @@
       </c>
       <c r="C117" s="22" t="inlineStr">
         <is>
-          <t>XSPS01EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D117" s="22" t="inlineStr">
         <is>
-          <t>Porsche</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E117" s="22" t="inlineStr">
@@ -7285,27 +7277,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F117" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F117" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G117" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H117" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I117" s="26" t="n">
-        <v>18</v>
+        <v>49.99</v>
       </c>
       <c r="J117" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSPS01EN Porsche Style XM38 4Buttons Red</t>
+          <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K117" s="27" t="inlineStr">
@@ -7313,7 +7305,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L117" s="25" t="n"/>
+      <c r="L117" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="22" t="inlineStr">
@@ -7328,12 +7324,12 @@
       </c>
       <c r="C118" s="22" t="inlineStr">
         <is>
-          <t>XSSBR0EN</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="D118" s="22" t="inlineStr">
         <is>
-          <t>Subaru</t>
+          <t>Lexus</t>
         </is>
       </c>
       <c r="E118" s="22" t="inlineStr">
@@ -7341,27 +7337,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F118" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+      <c r="F118" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G118" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38 (TOY.T)</t>
         </is>
       </c>
       <c r="H118" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
         </is>
       </c>
       <c r="I118" s="26" t="n">
-        <v>18.5</v>
+        <v>52</v>
       </c>
       <c r="J118" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSSBR0EN Subaru Style XM38 4Buttons</t>
+          <t>Xhorse Lexus Smart Key 315/433MHz 4Buttons XSTO01EN</t>
         </is>
       </c>
       <c r="K118" s="27" t="inlineStr">
@@ -7369,7 +7365,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L118" s="25" t="n"/>
+      <c r="L118" s="25" t="inlineStr">
+        <is>
+          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="22" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="C119" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSTO03EN</t>
         </is>
       </c>
       <c r="D119" s="22" t="inlineStr">
@@ -7413,11 +7413,11 @@
         </is>
       </c>
       <c r="I119" s="26" t="n">
-        <v>39.99</v>
+        <v>40</v>
       </c>
       <c r="J119" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Toyota XM38 Smart Key 4Buttons Support 4D 8A 4A All in One With Key Shell XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSTO03EN Toyota Style XM38 4Buttons</t>
         </is>
       </c>
       <c r="K119" s="27" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="L119" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+          <t>판매처마다 말이 달라 확인이 필요해요. [근거] key4는 "공용 폴딩 키날을 구매하라"고 안내. 반면 같은 XM38 토요타 모양(XSTO01EN)은 ABKEYS가 토요타 스마트키용 비상키(TOY48)를 지정. 모양이 토요타 스마트키형이라 TOY48 비상키일 가능성이 높음</t>
         </is>
       </c>
     </row>
@@ -7439,17 +7439,17 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>4버튼</t>
+          <t>5버튼</t>
         </is>
       </c>
       <c r="C120" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSCD01EN</t>
         </is>
       </c>
       <c r="D120" s="22" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Cadillac</t>
         </is>
       </c>
       <c r="E120" s="22" t="inlineStr">
@@ -7457,27 +7457,27 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F120" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F120" s="28" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G120" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H120" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I120" s="26" t="n">
-        <v>47</v>
+        <v>12.95</v>
       </c>
       <c r="J120" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons SUV XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSCD01EN Cadillac Style XM38 5Buttons</t>
         </is>
       </c>
       <c r="K120" s="27" t="inlineStr">
@@ -7485,11 +7485,7 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L120" s="25" t="inlineStr">
-        <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
-        </is>
-      </c>
+      <c r="L120" s="25" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="22" t="inlineStr">
@@ -7499,17 +7495,17 @@
       </c>
       <c r="B121" s="23" t="inlineStr">
         <is>
-          <t>4버튼</t>
+          <t>5버튼</t>
         </is>
       </c>
       <c r="C121" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSJP01EN</t>
         </is>
       </c>
       <c r="D121" s="22" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Jeep</t>
         </is>
       </c>
       <c r="E121" s="22" t="inlineStr">
@@ -7524,20 +7520,20 @@
       </c>
       <c r="G121" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H121" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I121" s="26" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="J121" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSJP01EN Jeep Style XM38 5Buttons</t>
         </is>
       </c>
       <c r="K121" s="27" t="inlineStr">
@@ -7547,7 +7543,7 @@
       </c>
       <c r="L121" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+          <t>비상키가 들어 있는 제품이라 키날을 따로 살 필요가 없어요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 키 규격 CY22. 단 같은 페이지 안내문에는 "키날 미포함"이라는 문구도 있어 판매처에 확인 권장</t>
         </is>
       </c>
     </row>
@@ -7559,17 +7555,17 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>4버튼</t>
+          <t>5버튼</t>
         </is>
       </c>
       <c r="C122" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSLR01EN</t>
         </is>
       </c>
       <c r="D122" s="22" t="inlineStr">
         <is>
-          <t>Lexus</t>
+          <t>Rover</t>
         </is>
       </c>
       <c r="E122" s="22" t="inlineStr">
@@ -7584,20 +7580,20 @@
       </c>
       <c r="G122" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (범용)</t>
         </is>
       </c>
       <c r="H122" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
         </is>
       </c>
       <c r="I122" s="26" t="n">
-        <v>49</v>
+        <v>18.5</v>
       </c>
       <c r="J122" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Lexus Smart Key 315/433MHz 4Buttons XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSLR01EN Land Rover Style XM38 5Buttons</t>
         </is>
       </c>
       <c r="K122" s="27" t="inlineStr">
@@ -7607,7 +7603,7 @@
       </c>
       <c r="L122" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+          <t>랜드로버 스마트키 모양이라 랜드로버 스마트키용 비상키(HU101 규격)를 끼우는 것으로 보여요. [근거] ABKEYS가 "Range Rover, Land Rover 2010+ Smart Key Blade, HU101"을 지정, 3D Group도 "Blade Reference HU101". 단 key4는 공용 폴딩 키날 구매를 안내해서 판매처마다 말이 달라요 → 구매 전 확인 필요</t>
         </is>
       </c>
     </row>
@@ -7619,17 +7615,17 @@
       </c>
       <c r="B123" s="23" t="inlineStr">
         <is>
-          <t>4버튼</t>
+          <t>5버튼</t>
         </is>
       </c>
       <c r="C123" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSLR03EN</t>
         </is>
       </c>
       <c r="D123" s="22" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Rover</t>
         </is>
       </c>
       <c r="E123" s="22" t="inlineStr">
@@ -7644,20 +7640,20 @@
       </c>
       <c r="G123" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H123" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I123" s="26" t="n">
-        <v>49</v>
+        <v>19.25</v>
       </c>
       <c r="J123" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
+          <t>Xhorse Universal Smart Key XSLR03EN Land Rover Style For NXP Chip 5Buttons</t>
         </is>
       </c>
       <c r="K123" s="27" t="inlineStr">
@@ -7667,7 +7663,7 @@
       </c>
       <c r="L123" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+          <t>키날 정보를 적은 판매처를 찾지 못했어요. [근거] Locksmith Keyless 등 설명에 키날 언급 없음. 같은 랜드로버 모양(XSLR01EN)은 ABKEYS가 랜드로버 스마트키용 비상키(HU101)를 지정 → 같은 방식일 가능성이 높지만 확인 필요</t>
         </is>
       </c>
     </row>
@@ -7679,22 +7675,18 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>4버튼</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="C124" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
-        </is>
-      </c>
-      <c r="D124" s="22" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
+          <t>XSBTK0EN</t>
+        </is>
+      </c>
+      <c r="D124" s="22" t="inlineStr"/>
       <c r="E124" s="22" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>블루투스 디지털 키</t>
         </is>
       </c>
       <c r="F124" s="24" t="inlineStr">
@@ -7704,20 +7696,20 @@
       </c>
       <c r="G124" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="H124" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="I124" s="26" t="n">
-        <v>49.99</v>
+        <v>80</v>
       </c>
       <c r="J124" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Toyota Smart Key 315/433MHz 4Buttons XSTO01EN</t>
+          <t>Xhorse Bluetooth Digital Smart Key XSBTK0EN Supports iOS Android - Turn your Phone to a Car Key</t>
         </is>
       </c>
       <c r="K124" s="27" t="inlineStr">
@@ -7727,7 +7719,7 @@
       </c>
       <c r="L124" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
         </is>
       </c>
     </row>
@@ -7739,22 +7731,18 @@
       </c>
       <c r="B125" s="23" t="inlineStr">
         <is>
-          <t>4버튼</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="C125" s="22" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
-        </is>
-      </c>
-      <c r="D125" s="22" t="inlineStr">
-        <is>
-          <t>Lexus</t>
-        </is>
-      </c>
+          <t>XSWK02EN</t>
+        </is>
+      </c>
+      <c r="D125" s="22" t="inlineStr"/>
       <c r="E125" s="22" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트워치형 키</t>
         </is>
       </c>
       <c r="F125" s="24" t="inlineStr">
@@ -7764,20 +7752,20 @@
       </c>
       <c r="G125" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="H125" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="I125" s="26" t="n">
-        <v>52</v>
+        <v>139.3</v>
       </c>
       <c r="J125" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Lexus Smart Key 315/433MHz 4Buttons XSTO01EN</t>
+          <t>Xhorse Smart Watch Wearable Super Car Key Midnight Black SW-007 XSWK02EN</t>
         </is>
       </c>
       <c r="K125" s="27" t="inlineStr">
@@ -7787,7 +7775,7 @@
       </c>
       <c r="L125" s="25" t="inlineStr">
         <is>
-          <t>토요타·렉서스 순정 스마트키와 같은 모양이라, 폴딩 키날이 아니라 토요타·렉서스 스마트키에 꽂는 납작한 비상키(TOY48 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Toyota/Lexus Smart Key Blade 69515-xxxxx, TOY48"을 지정(쉘 모양별로 품번 다름). Honrow도 이 쉘 전용 비상키(A/B/C 타입)를 따로 판매</t>
+          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
         </is>
       </c>
     </row>
@@ -7799,22 +7787,18 @@
       </c>
       <c r="B126" s="23" t="inlineStr">
         <is>
-          <t>4버튼</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="C126" s="22" t="inlineStr">
         <is>
-          <t>XSTO03EN</t>
-        </is>
-      </c>
-      <c r="D126" s="22" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
+          <t>XSWK05EN</t>
+        </is>
+      </c>
+      <c r="D126" s="22" t="inlineStr"/>
       <c r="E126" s="22" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트워치형 키</t>
         </is>
       </c>
       <c r="F126" s="24" t="inlineStr">
@@ -7824,20 +7808,20 @@
       </c>
       <c r="G126" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="H126" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="I126" s="26" t="n">
-        <v>40</v>
+        <v>199</v>
       </c>
       <c r="J126" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSTO03EN Toyota Style XM38 4Buttons</t>
+          <t>Xhorse Smart Watch Wearable Super Car Key Navy Blue SW-007 XSWK05EN</t>
         </is>
       </c>
       <c r="K126" s="27" t="inlineStr">
@@ -7847,7 +7831,7 @@
       </c>
       <c r="L126" s="25" t="inlineStr">
         <is>
-          <t>판매처마다 말이 달라 확인이 필요해요. [근거] key4는 "공용 폴딩 키날을 구매하라"고 안내. 반면 같은 XM38 토요타 모양(XSTO01EN)은 ABKEYS가 토요타 스마트키용 비상키(TOY48)를 지정. 모양이 토요타 스마트키형이라 TOY48 비상키일 가능성이 높음</t>
+          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
         </is>
       </c>
     </row>
@@ -7859,45 +7843,45 @@
       </c>
       <c r="B127" s="23" t="inlineStr">
         <is>
-          <t>5버튼</t>
+          <t>3버튼</t>
         </is>
       </c>
       <c r="C127" s="22" t="inlineStr">
         <is>
-          <t>XSCD01EN</t>
+          <t>XSMA41EN</t>
         </is>
       </c>
       <c r="D127" s="22" t="inlineStr">
         <is>
-          <t>Cadillac</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="E127" s="22" t="inlineStr">
         <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="F127" s="28" t="inlineStr">
-        <is>
-          <t>O</t>
+          <t>스마트키 기판 (XS)</t>
+        </is>
+      </c>
+      <c r="F127" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
       <c r="G127" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="H127" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="I127" s="26" t="n">
-        <v>12.95</v>
+        <v>34.99</v>
       </c>
       <c r="J127" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSCD01EN Cadillac Style XM38 5Buttons</t>
+          <t>Xhorse XSMA41EN Smart Key Board With 3Buttons for Audi MLB Cars</t>
         </is>
       </c>
       <c r="K127" s="27" t="inlineStr">
@@ -7905,7 +7889,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="L127" s="25" t="n"/>
+      <c r="L127" s="25" t="inlineStr">
+        <is>
+          <t>[XS 기판] XZ처럼 기판만 파는 제품이지만 XS 범용 스마트키 제품군이에요. XZ와 달리 "특정 브랜드만 생성 가능"이라는 제한 표기가 없고, 판매처 설명상 아우디·폭스바겐·벤틀리·포르쉐·람보르기니 MLB 차량을 지원해요 (Xhorse MLB 장비 필요, 칩 종류는 판매처에 명시 없음). / 아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="22" t="inlineStr">
@@ -7915,22 +7903,22 @@
       </c>
       <c r="B128" s="23" t="inlineStr">
         <is>
-          <t>5버튼</t>
+          <t>3버튼</t>
         </is>
       </c>
       <c r="C128" s="22" t="inlineStr">
         <is>
-          <t>XSJP01EN</t>
+          <t>XSMA4YEN</t>
         </is>
       </c>
       <c r="D128" s="22" t="inlineStr">
         <is>
-          <t>Jeep</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="E128" s="22" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="F128" s="24" t="inlineStr">
@@ -7940,20 +7928,20 @@
       </c>
       <c r="G128" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="H128" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="I128" s="26" t="n">
-        <v>19</v>
+        <v>38.99</v>
       </c>
       <c r="J128" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSJP01EN Jeep Style XM38 5Buttons</t>
+          <t>Xhorse XSMA4YEN Smart Key Board With 3Buttons for Audi A4 MLB Cars Works with Xhorse MLB Tool</t>
         </is>
       </c>
       <c r="K128" s="27" t="inlineStr">
@@ -7963,7 +7951,7 @@
       </c>
       <c r="L128" s="25" t="inlineStr">
         <is>
-          <t>비상키가 들어 있는 제품이라 키날을 따로 살 필요가 없어요. [근거] ABKEYS 상품 정보 "Key Blade: Included", 키 규격 CY22. 단 같은 페이지 안내문에는 "키날 미포함"이라는 문구도 있어 판매처에 확인 권장</t>
+          <t>[XS 기판] XZ처럼 기판만 파는 제품이지만 XS 범용 스마트키 제품군이에요. XZ와 달리 "특정 브랜드만 생성 가능"이라는 제한 표기가 없고, 판매처 설명상 아우디·폭스바겐·벤틀리·포르쉐·람보르기니 MLB 차량을 지원해요 (Xhorse MLB 장비 필요, 칩 종류는 판매처에 명시 없음). / 아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
         </is>
       </c>
     </row>
@@ -7975,22 +7963,22 @@
       </c>
       <c r="B129" s="23" t="inlineStr">
         <is>
-          <t>5버튼</t>
+          <t>3버튼</t>
         </is>
       </c>
       <c r="C129" s="22" t="inlineStr">
         <is>
-          <t>XSLR01EN</t>
+          <t>XSMA8YEN</t>
         </is>
       </c>
       <c r="D129" s="22" t="inlineStr">
         <is>
-          <t>Rover</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="E129" s="22" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="F129" s="24" t="inlineStr">
@@ -8000,20 +7988,20 @@
       </c>
       <c r="G129" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="H129" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="I129" s="26" t="n">
-        <v>18.5</v>
+        <v>38.99</v>
       </c>
       <c r="J129" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSLR01EN Land Rover Style XM38 5Buttons</t>
+          <t>Xhorse XSMA8YEN Smart Key Board With 3Buttons for Audi A8 MLB Cars Works with Xhorse MLB Tool</t>
         </is>
       </c>
       <c r="K129" s="27" t="inlineStr">
@@ -8023,7 +8011,7 @@
       </c>
       <c r="L129" s="25" t="inlineStr">
         <is>
-          <t>랜드로버 스마트키 모양이라 랜드로버 스마트키용 비상키(HU101 규격)를 끼우는 것으로 보여요. [근거] ABKEYS가 "Range Rover, Land Rover 2010+ Smart Key Blade, HU101"을 지정, 3D Group도 "Blade Reference HU101". 단 key4는 공용 폴딩 키날 구매를 안내해서 판매처마다 말이 달라요 → 구매 전 확인 필요</t>
+          <t>[XS 기판] XZ처럼 기판만 파는 제품이지만 XS 범용 스마트키 제품군이에요. XZ와 달리 "특정 브랜드만 생성 가능"이라는 제한 표기가 없고, 판매처 설명상 아우디·폭스바겐·벤틀리·포르쉐·람보르기니 MLB 차량을 지원해요 (Xhorse MLB 장비 필요, 칩 종류는 판매처에 명시 없음). / 아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
         </is>
       </c>
     </row>
@@ -8035,22 +8023,22 @@
       </c>
       <c r="B130" s="23" t="inlineStr">
         <is>
-          <t>5버튼</t>
+          <t>3버튼</t>
         </is>
       </c>
       <c r="C130" s="22" t="inlineStr">
         <is>
-          <t>XSLR03EN</t>
+          <t>XSMPSYEN</t>
         </is>
       </c>
       <c r="D130" s="22" t="inlineStr">
         <is>
-          <t>Rover</t>
+          <t>Porsche</t>
         </is>
       </c>
       <c r="E130" s="22" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="F130" s="24" t="inlineStr">
@@ -8060,20 +8048,20 @@
       </c>
       <c r="G130" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="H130" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>미기재</t>
         </is>
       </c>
       <c r="I130" s="26" t="n">
-        <v>19.25</v>
+        <v>38.99</v>
       </c>
       <c r="J130" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Key XSLR03EN Land Rover Style For NXP Chip 5Buttons</t>
+          <t>Xhorse XSMPSYEN Smart Key Board With 3Buttons for Porsche MLB Cars Works with Xhorse MLB Tool</t>
         </is>
       </c>
       <c r="K130" s="27" t="inlineStr">
@@ -8083,7 +8071,7 @@
       </c>
       <c r="L130" s="25" t="inlineStr">
         <is>
-          <t>키날 정보를 적은 판매처를 찾지 못했어요. [근거] Locksmith Keyless 등 설명에 키날 언급 없음. 같은 랜드로버 모양(XSLR01EN)은 ABKEYS가 랜드로버 스마트키용 비상키(HU101)를 지정 → 같은 방식일 가능성이 높지만 확인 필요</t>
+          <t>[XS 기판] XZ처럼 기판만 파는 제품이지만 XS 범용 스마트키 제품군이에요. XZ와 달리 "특정 브랜드만 생성 가능"이라는 제한 표기가 없고, 판매처 설명상 아우디·폭스바겐·벤틀리·포르쉐·람보르기니 MLB 차량을 지원해요 (Xhorse MLB 장비 필요, 칩 종류는 판매처에 명시 없음). / 아우디·포르쉐 순정 스마트키 모양의 기판이라, 아우디·포르쉐 스마트키용 비상키(HU162 규격)를 끼워야 해요. [근거] ABKEYS가 맞는 부품으로 "Audi Smart Key Blade, HU162" / "Porsche Smart Key Blade, HU162"를 지정</t>
         </is>
       </c>
     </row>
@@ -8095,18 +8083,22 @@
       </c>
       <c r="B131" s="23" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>4버튼</t>
         </is>
       </c>
       <c r="C131" s="22" t="inlineStr">
         <is>
-          <t>XSBTK0EN</t>
-        </is>
-      </c>
-      <c r="D131" s="22" t="inlineStr"/>
+          <t>XSADJ1EN</t>
+        </is>
+      </c>
+      <c r="D131" s="22" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
       <c r="E131" s="22" t="inlineStr">
         <is>
-          <t>블루투스 디지털 키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="F131" s="24" t="inlineStr">
@@ -8125,11 +8117,11 @@
         </is>
       </c>
       <c r="I131" s="26" t="n">
-        <v>80</v>
+        <v>44.99</v>
       </c>
       <c r="J131" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Bluetooth Digital Smart Key XSBTK0EN Supports iOS Android - Turn your Phone to a Car Key</t>
+          <t>Xhorse Universal Smart Key For Audi 315MHz 433MHz 868MHz 4Buttons XSADJ1EN</t>
         </is>
       </c>
       <c r="K131" s="27" t="inlineStr">
@@ -8139,7 +8131,7 @@
       </c>
       <c r="L131" s="25" t="inlineStr">
         <is>
-          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
+          <t>[XS 기판] XZ처럼 기판만 파는 제품이지만 XS 범용 스마트키 제품군이에요. XZ와 달리 "특정 브랜드만 생성 가능"이라는 제한 표기가 없어요 (단, 다른 브랜드 등록이 되는지는 판매처에 명시 없음). / 아우디 순정 스마트키(2008~2016 A4·A5·A6·A7·A8·Q5) 케이스에 넣는 기판만 파는 제품이에요. 비상키는 그 아우디 케이스에 맞는 것을 써야 해요. [근거] UHS: "Board only(기판만)", "Emergency Blade (not included)", 적용 차종 목록</t>
         </is>
       </c>
     </row>
@@ -8151,18 +8143,22 @@
       </c>
       <c r="B132" s="23" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>4버튼</t>
         </is>
       </c>
       <c r="C132" s="22" t="inlineStr">
         <is>
-          <t>XSWK02EN</t>
-        </is>
-      </c>
-      <c r="D132" s="22" t="inlineStr"/>
+          <t>XSBMB1EN</t>
+        </is>
+      </c>
+      <c r="D132" s="22" t="inlineStr">
+        <is>
+          <t>Bread</t>
+        </is>
+      </c>
       <c r="E132" s="22" t="inlineStr">
         <is>
-          <t>스마트워치형 키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="F132" s="24" t="inlineStr">
@@ -8181,11 +8177,11 @@
         </is>
       </c>
       <c r="I132" s="26" t="n">
-        <v>139.3</v>
+        <v>19.99</v>
       </c>
       <c r="J132" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Smart Watch Wearable Super Car Key Midnight Black SW-007 XSWK02EN</t>
+          <t>Xhorse XSBMB1EN BMW Smart Key PCB BMW Bread Style for F/G Chassis BDC2 BDC3 4Buttons</t>
         </is>
       </c>
       <c r="K132" s="27" t="inlineStr">
@@ -8195,7 +8191,7 @@
       </c>
       <c r="L132" s="25" t="inlineStr">
         <is>
-          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
+          <t>[XS 기판] XZ처럼 기판만 파는 제품이지만 XS 범용 스마트키 제품군이에요. 판매처 표기상 XS 스마트키와 같은 XM38 칩이 들어 있고, XZ와 달리 "특정 브랜드만 생성 가능"이라는 제한 표기가 없어요 (단, 다른 브랜드 등록이 되는지는 판매처에 명시 없음). / BMW 스마트키용 기판만 파는 제품이에요(쉘·키날·배터리 없음). 비상키는 기판을 넣을 BMW 쉘에 맞는 것을 따로 준비해야 해요. [근거] ABKEYS: "PCB board only, No shell included, Key blade is not included"</t>
         </is>
       </c>
     </row>
@@ -8207,18 +8203,22 @@
       </c>
       <c r="B133" s="23" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>4버튼</t>
         </is>
       </c>
       <c r="C133" s="22" t="inlineStr">
         <is>
-          <t>XSWK05EN</t>
-        </is>
-      </c>
-      <c r="D133" s="22" t="inlineStr"/>
+          <t>XSBMU1EN</t>
+        </is>
+      </c>
+      <c r="D133" s="22" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
       <c r="E133" s="22" t="inlineStr">
         <is>
-          <t>스마트워치형 키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="F133" s="24" t="inlineStr">
@@ -8237,11 +8237,11 @@
         </is>
       </c>
       <c r="I133" s="26" t="n">
-        <v>199</v>
+        <v>19.99</v>
       </c>
       <c r="J133" s="25" t="inlineStr">
         <is>
-          <t>Xhorse Smart Watch Wearable Super Car Key Navy Blue SW-007 XSWK05EN</t>
+          <t>Xhorse XSBMU1EN BMW Smart Key PCB BMW U Style for F/G Chassis BDC2 BDC3 4Buttons</t>
         </is>
       </c>
       <c r="K133" s="27" t="inlineStr">
@@ -8251,7 +8251,7 @@
       </c>
       <c r="L133" s="25" t="inlineStr">
         <is>
-          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
+          <t>[XS 기판] XZ처럼 기판만 파는 제품이지만 XS 범용 스마트키 제품군이에요. 판매처 표기상 XS 스마트키와 같은 XM38 칩이 들어 있고, XZ와 달리 "특정 브랜드만 생성 가능"이라는 제한 표기가 없어요 (단, 다른 브랜드 등록이 되는지는 판매처에 명시 없음). / BMW 스마트키용 기판만 파는 제품이에요(쉘·키날·배터리 없음). 비상키는 기판을 넣을 BMW 쉘에 맞는 것을 따로 준비해야 해요. [근거] ABKEYS: "PCB board only, No shell included, Key blade is not included"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit chip and transponder columns against multiple sellers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -4748,12 +4748,12 @@
       </c>
       <c r="G73" s="16" t="inlineStr">
         <is>
-          <t>XT27 슈퍼칩 (A/B 버전 미기재)</t>
+          <t>XT27A 슈퍼칩</t>
         </is>
       </c>
       <c r="H73" s="19" t="inlineStr">
         <is>
-          <t>XT27A: 11, 12, 13, 7935, 7936, 46, 47, 48, 4C, 4D, 4E, 8A, 8C, 8E / XT27B: +49, 4A, MQB48</t>
+          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
         </is>
       </c>
       <c r="I73" s="20" t="n">
@@ -4804,12 +4804,12 @@
       </c>
       <c r="G74" s="16" t="inlineStr">
         <is>
-          <t>XT27 슈퍼칩 (A/B 버전 미기재)</t>
+          <t>XT27A 슈퍼칩</t>
         </is>
       </c>
       <c r="H74" s="19" t="inlineStr">
         <is>
-          <t>XT27A: 11, 12, 13, 7935, 7936, 46, 47, 48, 4C, 4D, 4E, 8A, 8C, 8E / XT27B: +49, 4A, MQB48</t>
+          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
         </is>
       </c>
       <c r="I74" s="20" t="n">
@@ -4860,12 +4860,12 @@
       </c>
       <c r="G75" s="16" t="inlineStr">
         <is>
-          <t>XT27 슈퍼칩 (A/B 버전 미기재)</t>
+          <t>XT27 슈퍼칩 (A/B 미기재)</t>
         </is>
       </c>
       <c r="H75" s="19" t="inlineStr">
         <is>
-          <t>XT27A: 11, 12, 13, 7935, 7936, 46, 47, 48, 4C, 4D, 4E, 8A, 8C, 8E / XT27B: +49, 4A, MQB48</t>
+          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13 (XT27B면 4A, MQB48 추가)</t>
         </is>
       </c>
       <c r="I75" s="20" t="n">
@@ -4916,12 +4916,12 @@
       </c>
       <c r="G76" s="16" t="inlineStr">
         <is>
-          <t>XT27 슈퍼칩 (A/B 버전 미기재)</t>
+          <t>XT27 슈퍼칩 (A/B 미기재)</t>
         </is>
       </c>
       <c r="H76" s="19" t="inlineStr">
         <is>
-          <t>XT27A: 11, 12, 13, 7935, 7936, 46, 47, 48, 4C, 4D, 4E, 8A, 8C, 8E / XT27B: +49, 4A, MQB48</t>
+          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13 (XT27B면 4A, MQB48 추가)</t>
         </is>
       </c>
       <c r="I76" s="20" t="n">
@@ -4972,12 +4972,12 @@
       </c>
       <c r="G77" s="16" t="inlineStr">
         <is>
-          <t>XT27 슈퍼칩 (A/B 버전 미기재)</t>
+          <t>XT27 슈퍼칩 (A/B 미기재)</t>
         </is>
       </c>
       <c r="H77" s="19" t="inlineStr">
         <is>
-          <t>XT27A: 11, 12, 13, 7935, 7936, 46, 47, 48, 4C, 4D, 4E, 8A, 8C, 8E / XT27B: +49, 4A, MQB48</t>
+          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13 (XT27B면 4A, MQB48 추가)</t>
         </is>
       </c>
       <c r="I77" s="20" t="n">
@@ -5028,12 +5028,12 @@
       </c>
       <c r="G78" s="16" t="inlineStr">
         <is>
-          <t>XT27 슈퍼칩 (A/B 버전 미기재)</t>
+          <t>XT27A 슈퍼칩</t>
         </is>
       </c>
       <c r="H78" s="19" t="inlineStr">
         <is>
-          <t>XT27A: 11, 12, 13, 7935, 7936, 46, 47, 48, 4C, 4D, 4E, 8A, 8C, 8E / XT27B: +49, 4A, MQB48</t>
+          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
         </is>
       </c>
       <c r="I78" s="20" t="n">
@@ -5084,12 +5084,12 @@
       </c>
       <c r="G79" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38</t>
         </is>
       </c>
       <c r="H79" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>4D, 8A (BMW 오토바이)</t>
         </is>
       </c>
       <c r="I79" s="26" t="n">
@@ -5144,12 +5144,12 @@
       </c>
       <c r="G80" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H80" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I80" s="26" t="n">
@@ -5204,12 +5204,12 @@
       </c>
       <c r="G81" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H81" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I81" s="26" t="n">
@@ -5264,12 +5264,12 @@
       </c>
       <c r="G82" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H82" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I82" s="26" t="n">
@@ -5324,12 +5324,12 @@
       </c>
       <c r="G83" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H83" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I83" s="26" t="n">
@@ -5384,12 +5384,12 @@
       </c>
       <c r="G84" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H84" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I84" s="26" t="n">
@@ -5444,12 +5444,12 @@
       </c>
       <c r="G85" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H85" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I85" s="26" t="n">
@@ -5504,12 +5504,12 @@
       </c>
       <c r="G86" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H86" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I86" s="26" t="n">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="H87" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I87" s="26" t="n">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="H88" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I88" s="26" t="n">
@@ -5681,7 +5681,7 @@
       </c>
       <c r="H89" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I89" s="26" t="n">
@@ -5732,12 +5732,12 @@
       </c>
       <c r="G90" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H90" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I90" s="26" t="n">
@@ -5788,12 +5788,12 @@
       </c>
       <c r="G91" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H91" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I91" s="26" t="n">
@@ -5844,12 +5844,12 @@
       </c>
       <c r="G92" s="22" t="inlineStr">
         <is>
-          <t>XM38 (범용)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H92" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I92" s="26" t="n">
@@ -5900,12 +5900,12 @@
       </c>
       <c r="G93" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H93" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I93" s="26" t="n">
@@ -5960,12 +5960,12 @@
       </c>
       <c r="G94" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H94" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I94" s="26" t="n">
@@ -6020,12 +6020,12 @@
       </c>
       <c r="G95" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H95" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I95" s="26" t="n">
@@ -6080,12 +6080,12 @@
       </c>
       <c r="G96" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H96" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I96" s="26" t="n">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="H97" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 + 4D, 8A (토요타 전용 코드 제외)</t>
         </is>
       </c>
       <c r="I97" s="26" t="n">
@@ -6196,12 +6196,12 @@
       </c>
       <c r="G98" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>NXP 스마트키 칩 (추정, 일부 판매처는 XM38로 표기)</t>
         </is>
       </c>
       <c r="H98" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원) (XM38이면 4D, 8A 추가)</t>
         </is>
       </c>
       <c r="I98" s="26" t="n">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="H99" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I99" s="26" t="n">
@@ -6313,7 +6313,7 @@
       </c>
       <c r="H100" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I100" s="26" t="n">
@@ -6369,7 +6369,7 @@
       </c>
       <c r="H101" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 + 4D, 8A (토요타 전용 코드 제외)</t>
         </is>
       </c>
       <c r="I101" s="26" t="n">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="H102" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 + 4D, 8A (토요타 전용 코드 제외)</t>
         </is>
       </c>
       <c r="I102" s="26" t="n">
@@ -6477,7 +6477,7 @@
       </c>
       <c r="H103" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I103" s="26" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="H104" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I104" s="26" t="n">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="H105" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I105" s="26" t="n">
@@ -6649,7 +6649,7 @@
       </c>
       <c r="H106" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I106" s="26" t="n">
@@ -6705,7 +6705,7 @@
       </c>
       <c r="H107" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I107" s="26" t="n">
@@ -6761,7 +6761,7 @@
       </c>
       <c r="H108" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I108" s="26" t="n">
@@ -6812,12 +6812,12 @@
       </c>
       <c r="G109" s="22" t="inlineStr">
         <is>
-          <t>NXP 스마트키 칩</t>
+          <t>NXP 스마트키 칩 (추정)</t>
         </is>
       </c>
       <c r="H109" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원) (추정)</t>
         </is>
       </c>
       <c r="I109" s="26" t="n">
@@ -6877,7 +6877,7 @@
       </c>
       <c r="H110" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 + 4D, 8A (토요타 전용 코드 제외)</t>
         </is>
       </c>
       <c r="I110" s="26" t="n">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="H111" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 + 4D, 8A (토요타 전용 코드 제외)</t>
         </is>
       </c>
       <c r="I111" s="26" t="n">
@@ -6984,12 +6984,12 @@
       </c>
       <c r="G112" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H112" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I112" s="26" t="n">
@@ -7044,12 +7044,12 @@
       </c>
       <c r="G113" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H113" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I113" s="26" t="n">
@@ -7104,12 +7104,12 @@
       </c>
       <c r="G114" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H114" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I114" s="26" t="n">
@@ -7164,12 +7164,12 @@
       </c>
       <c r="G115" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H115" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I115" s="26" t="n">
@@ -7224,12 +7224,12 @@
       </c>
       <c r="G116" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H116" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I116" s="26" t="n">
@@ -7284,12 +7284,12 @@
       </c>
       <c r="G117" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H117" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I117" s="26" t="n">
@@ -7344,12 +7344,12 @@
       </c>
       <c r="G118" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H118" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I118" s="26" t="n">
@@ -7404,12 +7404,12 @@
       </c>
       <c r="G119" s="22" t="inlineStr">
         <is>
-          <t>XM38 (TOY.T)</t>
+          <t>XM38 (토요타형)</t>
         </is>
       </c>
       <c r="H119" s="25" t="inlineStr">
         <is>
-          <t>NXP 스마트키 지원 칩 + 4D, 8A, 4A (토요타 포함)</t>
+          <t>토요타 4D (94·98·D4·9F·34 등), 8A (88·A8·A9·AA 등), 4A + NXP 스마트키 지원 칩</t>
         </is>
       </c>
       <c r="I119" s="26" t="n">
@@ -7469,7 +7469,7 @@
       </c>
       <c r="H120" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 + 4D, 8A (토요타 전용 코드 제외)</t>
         </is>
       </c>
       <c r="I120" s="26" t="n">
@@ -7525,7 +7525,7 @@
       </c>
       <c r="H121" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 + 4D, 8A (토요타 전용 코드 제외)</t>
         </is>
       </c>
       <c r="I121" s="26" t="n">
@@ -7585,7 +7585,7 @@
       </c>
       <c r="H122" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 + 4D, 8A (토요타 제외)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 + 4D, 8A (토요타 전용 코드 제외)</t>
         </is>
       </c>
       <c r="I122" s="26" t="n">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="H123" s="25" t="inlineStr">
         <is>
-          <t>46, 47, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I123" s="26" t="n">
@@ -7696,12 +7696,12 @@
       </c>
       <c r="G124" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>XM38 (UHS 표기)</t>
         </is>
       </c>
       <c r="H124" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>세부 목록 미기재 (판매처: 키리스 시동 차량 90% 이상 지원)</t>
         </is>
       </c>
       <c r="I124" s="26" t="n">
@@ -7752,12 +7752,12 @@
       </c>
       <c r="G125" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H125" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I125" s="26" t="n">
@@ -7808,12 +7808,12 @@
       </c>
       <c r="G126" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>NXP 스마트키 칩</t>
         </is>
       </c>
       <c r="H126" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 48, 49, 4A, MQB48, MQB49 (4D·8A 미지원)</t>
         </is>
       </c>
       <c r="I126" s="26" t="n">
@@ -7868,12 +7868,12 @@
       </c>
       <c r="G127" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>ID5A 49 칩 (UHS·ABKEYS·vvdishop 표기)</t>
         </is>
       </c>
       <c r="H127" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>ID49 계열 (아우디·폭스바겐·벤틀리·포르쉐·람보르기니 MLB)</t>
         </is>
       </c>
       <c r="I127" s="26" t="n">
@@ -7928,12 +7928,12 @@
       </c>
       <c r="G128" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>OEM 칩 (xhorseshop.eu: New Version OEM Chip)</t>
         </is>
       </c>
       <c r="H128" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>MLB 차량용 (칩 번호 미기재)</t>
         </is>
       </c>
       <c r="I128" s="26" t="n">
@@ -7993,7 +7993,7 @@
       </c>
       <c r="H129" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>MLB 차량용 (칩 번호 미기재)</t>
         </is>
       </c>
       <c r="I129" s="26" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H130" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>MLB 차량용 (칩 번호 미기재)</t>
         </is>
       </c>
       <c r="I130" s="26" t="n">
@@ -8108,12 +8108,12 @@
       </c>
       <c r="G131" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>트랜스폰더 내장 (종류 미기재)</t>
         </is>
       </c>
       <c r="H131" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>아우디 BCM2 (754J) 차량용 (칩 번호 미기재)</t>
         </is>
       </c>
       <c r="I131" s="26" t="n">
@@ -8168,12 +8168,12 @@
       </c>
       <c r="G132" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>XM38 (UHS 표기)</t>
         </is>
       </c>
       <c r="H132" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>BMW F/G 섀시 BDC2·BDC3·BCP용 (칩 번호 미기재)</t>
         </is>
       </c>
       <c r="I132" s="26" t="n">
@@ -8228,12 +8228,12 @@
       </c>
       <c r="G133" s="22" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>XM38 (UHS·MyKeySupply 표기)</t>
         </is>
       </c>
       <c r="H133" s="25" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>BMW F/G 섀시 BDC2·BDC3·BCP용 (칩 번호 미기재)</t>
         </is>
       </c>
       <c r="I133" s="26" t="n">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="H134" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I134" s="33" t="n">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="H136" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I136" s="33" t="n">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="H137" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I137" s="33" t="n">
@@ -8593,7 +8593,7 @@
       </c>
       <c r="H139" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I139" s="33" t="n">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="H140" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I140" s="33" t="n">
@@ -8713,7 +8713,7 @@
       </c>
       <c r="H141" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I141" s="33" t="n">
@@ -8773,7 +8773,7 @@
       </c>
       <c r="H142" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>4A (vvdishop 상품명 "Version 4 … 4A KeylessGo")</t>
         </is>
       </c>
       <c r="I142" s="33" t="n">
@@ -8893,7 +8893,7 @@
       </c>
       <c r="H144" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I144" s="33" t="n">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="H145" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I145" s="33" t="n">
@@ -9013,7 +9013,7 @@
       </c>
       <c r="H146" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I146" s="33" t="n">
@@ -9073,7 +9073,7 @@
       </c>
       <c r="H147" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I147" s="33" t="n">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="H148" s="32" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>미기재 (판매처 5곳 이상 확인, 칩 정보 없음)</t>
         </is>
       </c>
       <c r="I148" s="33" t="n">
@@ -9316,7 +9316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9446,10 +9446,22 @@
     <row r="11">
       <c r="A11" s="36" t="inlineStr">
         <is>
+          <t>내장 칩·지원 트랜스폰더 점검 (2026-09-30)</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>UHS, Locksmith Keyless, keyless-city, Best Key Supply, ABKEYS 등 판매처 5곳 이상의 모델별 설명으로 대조. XE는 판매처가 XT27A라고 밝힌 모델만 XT27A로 표기. XS는 NXP 스마트키 / XM38 범용 / XM38 토요타형으로 구분. "추정"·"미기재"는 모델별 근거가 없는 항목</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="36" t="inlineStr">
+        <is>
           <t>목록에 없는 모델</t>
         </is>
       </c>
-      <c r="B11" s="36" t="inlineStr">
+      <c r="B12" s="36" t="inlineStr">
         <is>
           <t>XT57B 2세대 XE(XEB520EN, XEKF30EN 등) 등은 ABKEYS에 없어 제외</t>
         </is>

</xml_diff>

<commit_message>
Fix XSMQB4EN chip list override
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -13309,12 +13309,12 @@
       </c>
       <c r="G187" s="20" t="inlineStr">
         <is>
-          <t>미기재 (XSMQB1EN 업그레이드 버전)</t>
+          <t>미기재 (XSMQB1EN의 업그레이드 버전)</t>
         </is>
       </c>
       <c r="H187" s="20" t="inlineStr">
         <is>
-          <t>미기재</t>
+          <t>46, 47, 48, 49, 4A, MQB (xhorseshop.eu 표기)</t>
         </is>
       </c>
       <c r="I187" s="23" t="n">

</xml_diff>

<commit_message>
Label flip-style XE/XK/XN remotes as folding keys; prefer in-stock prices
Nine rows that ABKEYS titles only as 'Super Remote'/'Remote' are sold as
Flip/Folding by other sellers. Adds XEFO21EN as the new version of
XEFO01EN and picks in-stock single prices before out-of-stock ones.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -999,21 +999,17 @@
         </is>
       </c>
       <c r="I6" s="5" t="n">
-        <v>9.449999999999999</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>6.27</v>
+      </c>
+      <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>xhorsestore.co.uk</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wire Flip Remote Key 2nd Generation Honda Style 3 Button XKHO22EN (New Version Of XKHO02EN)</t>
+          <t>XHORSE XKHO22EN for Honda Model (Foldable 2+1 Buttons) Second Generation Universal Remote Key</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -1279,21 +1275,17 @@
         </is>
       </c>
       <c r="I10" s="5" t="n">
-        <v>9.449999999999999</v>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>9.73</v>
+      </c>
+      <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wire Flip Remote Key 2nd Generation Toyota Style 2 Button XKTO21EN (New Version of XKTO01EN)</t>
+          <t>Xhorse - XKTO21EN - 2nd Generation w/ New XM5118 Chip Wire Remote Key Toyota Flip 2 Buttons (Replacement For XKTO01EN)</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
@@ -1350,21 +1342,21 @@
         </is>
       </c>
       <c r="I11" s="5" t="n">
-        <v>8.949999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>판매처 품절 표시</t>
+          <t>5개 묶음 $34.00 ÷ 5 · VVDIshop의 낱개 표기 가격 $36.99는 묶음 가격으로 보여 제외</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>OBDII365</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wired Remote Key 2nd Generation XKTO25EN (New Version of XKTO05EN)</t>
+          <t>[5Pcs/Set] XHORSE XKTO25EN for Toyota Models 2 Buttons Triangle Second Generation Wired Remote</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
@@ -1492,21 +1484,17 @@
         </is>
       </c>
       <c r="I13" s="5" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>11.76</v>
+      </c>
+      <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Royal Key Supply</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wired Remote Key 2nd Generation Audi Style XKA620EN</t>
+          <t>Xhorse - (2nd Gen) Universal Wire Remote Key 3B (XKA620EN) For VVDI</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -2276,21 +2264,17 @@
         </is>
       </c>
       <c r="I25" s="5" t="n">
-        <v>8.35</v>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>10.95</v>
+      </c>
+      <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wired Flip Remote 3 Button VW Style XKB520EN (New Version of XKB501EN)</t>
+          <t>Xhorse / XKB520EN / Volkswagen B5 Style / 3-Button Universal Remote Flip Key / For VVDI Key Tool (Wired) (Black) (Replacement For XKB501EN)</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
@@ -2686,21 +2670,17 @@
         </is>
       </c>
       <c r="I31" s="5" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>9.73</v>
+      </c>
+      <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wired Flip Remote Key 2nd Generation MQB Type 3 Button XKDM05EN XKMQB1EN (New Version of XKMQB1EN)</t>
+          <t>Xhorse / XKDM05EN / Volkswagen MQB Style / 3-Button Universal Remote Flip Key / For VVDI Key Tool (Wired) (Replacement For XKMQB1EN)</t>
         </is>
       </c>
       <c r="M31" s="6" t="inlineStr">
@@ -3691,21 +3671,17 @@
         </is>
       </c>
       <c r="I46" s="5" t="n">
-        <v>9.449999999999999</v>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>9.699999999999999</v>
+      </c>
+      <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wire Flip Remote Key 2nd Generation Honda Type 3 Button XKHO20EN (New Version of XKHO00EN)</t>
+          <t>Honda Style / XKHO20EN / 2nd Generation / 3-Button Universal Remote Flip Key for VVDI Key Tool (Wired) (Replacement For XKHO00EN)</t>
         </is>
       </c>
       <c r="M46" s="6" t="inlineStr">
@@ -4026,21 +4002,17 @@
         </is>
       </c>
       <c r="I51" s="5" t="n">
-        <v>8.35</v>
-      </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>8.5</v>
+      </c>
+      <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Keyless City</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wired Remote Key 2nd Generation Hyundai Style 3 Button XKHY20EN (New Version of XKHY00EN)</t>
+          <t>Xhorse - XKHY20EN - Hyundai / 3-Buttons Wired Remote Key</t>
         </is>
       </c>
       <c r="M51" s="6" t="inlineStr">
@@ -4101,21 +4073,17 @@
         </is>
       </c>
       <c r="I52" s="5" t="n">
-        <v>8.550000000000001</v>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>7.46</v>
+      </c>
+      <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Wire Remote Key 2nd Generation Hyundai Style 3+1 Button XKHY21EN (New Version of XKHY01EN)</t>
+          <t>Xhorse - XKHY21EN - 2nd Generation Wired Remote Key / Hyundai 4-Buttons w/ MX5118 Chip (Replacement For XKHY01EN)</t>
         </is>
       </c>
       <c r="M52" s="6" t="inlineStr">
@@ -4354,7 +4322,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -4440,21 +4408,17 @@
         </is>
       </c>
       <c r="I57" s="5" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="J57" s="2" t="n"/>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Wire Flip Remote Key 2nd Generation Knife Style 3 Button XKKF05EN (New Version of XKKF02EN)</t>
+          <t>Knife Style / - XKKF05EN - 3-Button Universal Remote Flip Key for VVDI Key Tool (Wired) (Replacement For XKKF02EN)</t>
         </is>
       </c>
       <c r="M57" s="6" t="inlineStr">
@@ -4563,7 +4527,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -5520,21 +5484,17 @@
         </is>
       </c>
       <c r="I73" s="5" t="n">
-        <v>9.449999999999999</v>
-      </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>10.5</v>
+      </c>
+      <c r="J73" s="2" t="n"/>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Royal Key Supply</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Wire Flip Remote Key 2nd Generation Toyota Style 3 Button XKTO20EN (New Version of XKTO00EN)</t>
+          <t>Xhorse - Toyota 2nd Gen Universal Wire Remote Key 3B (XKTO20EN) For VVDI</t>
         </is>
       </c>
       <c r="M73" s="6" t="inlineStr">
@@ -5666,21 +5626,17 @@
         </is>
       </c>
       <c r="I75" s="5" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>9.43</v>
+      </c>
+      <c r="J75" s="2" t="n"/>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Wire Remote 2nd Generation Toyota Style 3 Button XKTO24EN (New Version of XKTO04EN)</t>
+          <t>Xhorse - XKTO24EN - Toyota Style / 3-Button Universal Remote Head Key for VVDI Key Tools - XM5118 Chip - (Wireless) (Replacement For XKTO04EN)</t>
         </is>
       </c>
       <c r="M75" s="6" t="inlineStr">
@@ -5808,21 +5764,17 @@
         </is>
       </c>
       <c r="I77" s="5" t="n">
-        <v>9.65</v>
-      </c>
-      <c r="J77" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>13.05</v>
+      </c>
+      <c r="J77" s="2" t="n"/>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wire Remote Flip Key 2nd Generation Audi Style XKAU22EN (New Version of XKAU02EN)</t>
+          <t>Xhorse - XKAU22EN - Audi Style / 4-Button Universal Remote Key for VVDI Key Tool (Wired) (2nd Generation)</t>
         </is>
       </c>
       <c r="M77" s="6" t="inlineStr">
@@ -6080,21 +6032,17 @@
         </is>
       </c>
       <c r="I81" s="5" t="n">
-        <v>9.65</v>
-      </c>
-      <c r="J81" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>9.75</v>
+      </c>
+      <c r="J81" s="2" t="n"/>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Keyless City</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Wire Flip Remote Key 2nd Generation Buick Style 4 Button XKBU22EN (New Version of XKBU02EN)</t>
+          <t>Xhorse - XKBU22EN - 2nd Generation Wired Remote Key (Foldable 4 Buttons) Buick Flip / 4-Buttons w/ MX5118 Chip</t>
         </is>
       </c>
       <c r="M81" s="6" t="inlineStr">
@@ -6490,21 +6438,21 @@
         </is>
       </c>
       <c r="I87" s="5" t="n">
-        <v>9.949999999999999</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>판매처 품절 표시</t>
+          <t>5개 묶음 $44.80 ÷ 5 · xhorsestore.co.uk의 낱개 표기 가격 $44.80는 묶음 가격으로 보여 제외</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>xhorse.co.uk</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wired Remote Key 2nd Generation XKFEF8EN (New Version of XKFEF6EN )</t>
+          <t>Xhorse XKFEF8EN Universal Remote Key FA.LL Type Wired Folding Key 4 Buttons Bright Black 5PCS</t>
         </is>
       </c>
       <c r="M87" s="6" t="inlineStr">
@@ -6766,21 +6714,21 @@
         </is>
       </c>
       <c r="I91" s="5" t="n">
-        <v>8.949999999999999</v>
+        <v>6.6</v>
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>판매처 품절 표시</t>
+          <t>5개 묶음 $33.00 ÷ 5 · VVDIshop의 낱개 표기 가격 $35.99는 묶음 가격으로 보여 제외</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>OBDII365</t>
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wire Remote Key 2nd Generation Ford Style 4 Button XKFO22EN (New Version of XKFO02EN)</t>
+          <t>[5pcs/set] XHORSE XKFO22EN for Ford Models 4 Buttons Split Square Second Generation Wired Remote</t>
         </is>
       </c>
       <c r="M91" s="6" t="inlineStr">
@@ -7180,21 +7128,17 @@
         </is>
       </c>
       <c r="I97" s="5" t="n">
-        <v>8.35</v>
-      </c>
-      <c r="J97" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>8.529999999999999</v>
+      </c>
+      <c r="J97" s="2" t="n"/>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Royal Key Supply</t>
         </is>
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Wire Remote 2nd Generation Honda Style 5 Button XKHO23EN (New Version of XKHO03EN)</t>
+          <t>Xhorse - Honda Style Universal Wire Remote 5B (XKHO23EN) VVDI</t>
         </is>
       </c>
       <c r="M97" s="6" t="inlineStr">
@@ -7397,21 +7341,17 @@
         </is>
       </c>
       <c r="I100" s="5" t="n">
-        <v>8.65</v>
-      </c>
-      <c r="J100" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>9.949999999999999</v>
+      </c>
+      <c r="J100" s="2" t="n"/>
       <c r="K100" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wire Remote Key 2nd Generation Hyundai Style 4 Button XKHY24EN (New Version of XKHY04EN)</t>
+          <t>Xhorse - XKHY24EN - Universal Key Replacement For XKHY04EN / 4-Buttons Wired Remote Key</t>
         </is>
       </c>
       <c r="M100" s="6" t="inlineStr">
@@ -7744,21 +7684,17 @@
         </is>
       </c>
       <c r="I105" s="5" t="n">
-        <v>8.550000000000001</v>
-      </c>
-      <c r="J105" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>6.5</v>
+      </c>
+      <c r="J105" s="2" t="n"/>
       <c r="K105" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Royal Key Supply</t>
         </is>
       </c>
       <c r="L105" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wire Remote Key 2nd Generation 4 Button Nissan Type XKNI20EN (New Version of XKNI00EN)</t>
+          <t>Xhorse - Nissan Universal Wire Remote 4B Trunk (XKNI20EN)</t>
         </is>
       </c>
       <c r="M105" s="6" t="inlineStr">
@@ -8024,21 +7960,17 @@
         </is>
       </c>
       <c r="I109" s="5" t="n">
-        <v>9.449999999999999</v>
-      </c>
-      <c r="J109" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>12.98</v>
+      </c>
+      <c r="J109" s="2" t="n"/>
       <c r="K109" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Royal Key Supply</t>
         </is>
       </c>
       <c r="L109" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wired Flip Remote Key 2nd Generation 4 Button Toyota Style XKTO12EN (New Version of XKTO10EN)</t>
+          <t>Xhorse - Universal Wire Remote Key 4B 2nd Gen (XKTO12EN) For VVDI</t>
         </is>
       </c>
       <c r="M109" s="6" t="inlineStr">
@@ -8095,21 +8027,17 @@
         </is>
       </c>
       <c r="I110" s="5" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="J110" s="2" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>8.19</v>
+      </c>
+      <c r="J110" s="2" t="n"/>
       <c r="K110" s="2" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Royal Key Supply</t>
         </is>
       </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
-          <t>Xhorse Wire Remote 2nd Generation Toyota Style Triangle 4 Button XKTO22EN (New Version of XKTO02EN)</t>
+          <t>Xhorse - Toyota Style Universal Wire Remote Key 4B 2nd Gen (XKTO22EN) For VVDI</t>
         </is>
       </c>
       <c r="M110" s="6" t="inlineStr">
@@ -10086,21 +10014,17 @@
         </is>
       </c>
       <c r="I139" s="11" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="J139" s="8" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>11.95</v>
+      </c>
+      <c r="J139" s="8" t="n"/>
       <c r="K139" s="8" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L139" s="8" t="inlineStr">
         <is>
-          <t>Xhorse Universal Flip Wireless Remote Key 2nd Generation Honda Style XNHO20EN (New Version of XNHO00EN)</t>
+          <t>Xhorse / XNHO20EN / Honda Style / 3-Button Universal Remote Flip Key / For VVDI Key Tool (Wired)</t>
         </is>
       </c>
       <c r="M139" s="12" t="inlineStr">
@@ -10201,7 +10125,7 @@
       </c>
       <c r="E141" s="8" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F141" s="13" t="inlineStr">
@@ -10555,21 +10479,17 @@
         </is>
       </c>
       <c r="I146" s="11" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="J146" s="8" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>9.67</v>
+      </c>
+      <c r="J146" s="8" t="n"/>
       <c r="K146" s="8" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Royal Key Supply</t>
         </is>
       </c>
       <c r="L146" s="8" t="inlineStr">
         <is>
-          <t>Xhorse Universal Wireless Flip Remote Key 2nd Generation Toyota Style 3 Buttons XNTO20EN (New Version of XNTO00EN)</t>
+          <t>Xhorse - Universal Flip Key 3B (XNTO20EN) For VVDI (WIRELESS)</t>
         </is>
       </c>
       <c r="M146" s="12" t="inlineStr">
@@ -11501,21 +11421,17 @@
         </is>
       </c>
       <c r="I160" s="17" t="n">
-        <v>7.98</v>
-      </c>
-      <c r="J160" s="14" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="J160" s="14" t="n"/>
       <c r="K160" s="14" t="inlineStr">
         <is>
-          <t>UHS Hardware</t>
+          <t>Keyshop Online</t>
         </is>
       </c>
       <c r="L160" s="14" t="inlineStr">
         <is>
-          <t>VW Style XEB510EN / 3-Button Universal Remote Key - Built-in XT27B Super Chip</t>
+          <t>Xhorse Volkswagen B5 XT27B-Style Super Universal Flip Remote Key | 3-Buttons | VVDI | XEB510</t>
         </is>
       </c>
       <c r="M160" s="18" t="inlineStr">
@@ -11572,21 +11488,17 @@
         </is>
       </c>
       <c r="I161" s="17" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="J161" s="14" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>7.98</v>
+      </c>
+      <c r="J161" s="14" t="n"/>
       <c r="K161" s="14" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L161" s="14" t="inlineStr">
         <is>
-          <t>Xhorse Universal Super Remote Key 2nd Generation with New Chip XT57B VW Style XEB520EN (New Version of XEB510EN)</t>
+          <t>Xhorse - VW Style XEB520EN / 3-Button Universal Remote Key - Built-in XT27B Super Chip - 2nd Generation</t>
         </is>
       </c>
       <c r="M161" s="18" t="inlineStr">
@@ -11762,7 +11674,7 @@
       </c>
       <c r="E164" s="14" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F164" s="16" t="inlineStr">
@@ -11892,7 +11804,7 @@
       </c>
       <c r="E166" s="14" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F166" s="16" t="inlineStr">
@@ -12030,7 +11942,7 @@
       </c>
       <c r="E168" s="14" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F168" s="16" t="inlineStr">
@@ -12093,7 +12005,7 @@
       </c>
       <c r="E169" s="14" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F169" s="16" t="inlineStr">
@@ -12298,7 +12210,7 @@
       </c>
       <c r="E172" s="14" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F172" s="16" t="inlineStr">
@@ -12432,7 +12344,7 @@
       </c>
       <c r="E174" s="14" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F174" s="16" t="inlineStr">
@@ -12469,7 +12381,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="N174" s="14" t="n"/>
+      <c r="N174" s="14" t="inlineStr">
+        <is>
+          <t>신형: XEFO21EN</t>
+        </is>
+      </c>
       <c r="O174" s="14" t="n"/>
     </row>
     <row r="175">
@@ -12514,21 +12430,17 @@
         </is>
       </c>
       <c r="I175" s="17" t="n">
-        <v>12.35</v>
-      </c>
-      <c r="J175" s="14" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>8.949999999999999</v>
+      </c>
+      <c r="J175" s="14" t="n"/>
       <c r="K175" s="14" t="inlineStr">
         <is>
-          <t>Royal Key Supply</t>
+          <t>OBDII365</t>
         </is>
       </c>
       <c r="L175" s="14" t="inlineStr">
         <is>
-          <t>Xhorse - Universal Flip Key 4B (XEFO21EN) For VVDI</t>
+          <t>XHORSE XEFO21EN FOR.D Style Second Generation Super Remote Flip 4 Buttons</t>
         </is>
       </c>
       <c r="M175" s="18" t="inlineStr">
@@ -12536,7 +12448,11 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="N175" s="14" t="n"/>
+      <c r="N175" s="14" t="inlineStr">
+        <is>
+          <t>XEFO01EN의 신형</t>
+        </is>
+      </c>
       <c r="O175" s="14" t="n"/>
     </row>
     <row r="176">
@@ -12916,21 +12832,17 @@
         </is>
       </c>
       <c r="I181" s="23" t="n">
-        <v>65</v>
-      </c>
-      <c r="J181" s="20" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>75.52</v>
+      </c>
+      <c r="J181" s="20" t="n"/>
       <c r="K181" s="20" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>xhorsestore.co.uk</t>
         </is>
       </c>
       <c r="L181" s="20" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Flip Remote Key XM38 BMW Motorcycle XSBM90GL 3 Button</t>
+          <t>Xhorse XSBM90GL BMW Motorcycle XM38 Key for VVDI2 and Key Tool Plus</t>
         </is>
       </c>
       <c r="M181" s="24" t="inlineStr">
@@ -13054,21 +12966,17 @@
         </is>
       </c>
       <c r="I183" s="23" t="n">
-        <v>22.95</v>
-      </c>
-      <c r="J183" s="20" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>22.89</v>
+      </c>
+      <c r="J183" s="20" t="n"/>
       <c r="K183" s="20" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>UHS Hardware</t>
         </is>
       </c>
       <c r="L183" s="20" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Remote Key 2nd Generation MQB Style 3 Button XSDM04EN (New version of XSMQB1EN)</t>
+          <t>Xhorse - XSDM04EN MQB Type 3 Button Volkswagen - Smart Remote Replacing XSMQB1EN (PRE-ORDER)</t>
         </is>
       </c>
       <c r="M183" s="24" t="inlineStr">
@@ -15694,21 +15602,21 @@
         </is>
       </c>
       <c r="I223" s="23" t="n">
-        <v>44.95</v>
+        <v>38.9</v>
       </c>
       <c r="J223" s="20" t="inlineStr">
         <is>
-          <t>판매처 품절 표시</t>
+          <t>10개 묶음 $389.00 ÷ 10 · xhorse.co.uk의 낱개 표기 가격 $198.40는 묶음 가격으로 보여 제외</t>
         </is>
       </c>
       <c r="K223" s="20" t="inlineStr">
         <is>
-          <t>UHS Hardware</t>
+          <t>VVDIshop</t>
         </is>
       </c>
       <c r="L223" s="20" t="inlineStr">
         <is>
-          <t>Xhorse - XM Series Toyota 4D - 8A Rewritable Smart Key PCB - TOY.T XSTO00EN -  For VVDI2 - VVDI Key Tool - Mini - MAX - Plus Tablet</t>
+          <t>[10 Pieces] Xhorse Toyota 8A 4D Smart Key XSTO00EN XM28</t>
         </is>
       </c>
       <c r="M223" s="24" t="inlineStr">
@@ -16303,21 +16211,17 @@
         </is>
       </c>
       <c r="I232" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="J232" s="20" t="inlineStr">
-        <is>
-          <t>판매처 품절 표시</t>
-        </is>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="J232" s="20" t="n"/>
       <c r="K232" s="20" t="inlineStr">
         <is>
-          <t>Key4</t>
+          <t>Keyshop Online</t>
         </is>
       </c>
       <c r="L232" s="20" t="inlineStr">
         <is>
-          <t>Xhorse Universal Smart Proximity Remote For Audi 4 Button XSADJ1GL</t>
+          <t>2008-2019 Audi Smart Key 754J | 4-Buttons | 315/434/868MHz | XSADJ1GL (Xhorse-Aftermarket)</t>
         </is>
       </c>
       <c r="M232" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Re-check unconfirmed blade/chip rows against Xhorse product photos; label card keys
Xhorse accessory photos on dealer pages settle blade use for XNSZ01EN,
XNSZ02EN, XNFO00EN, XSLR01EN, XSLR03EN (universal blade) and XKHY20EN
(separate fob). Records XM38 for the new XS styles, XSCLN1EN's
'Transponder: NO' spec conflict, and marks King Card rows as card keys.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -152,7 +152,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -161,7 +161,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>키날 없이 버튼만 있는 분리형 리모컨이에요(문 잠금·해제용). [근거] xhorsetool.com 상품명 "Hyundai Separate 3 Buttons", 1세대 XKHY00EN도 같은 판매처에서 "Separate". 단, UHS·Keyless City 설명에는 "Flip"이라고 적혀 있어 판매처끼리 다름 (확인 필요)</t>
+          <t>키날 없이 버튼만 있는 분리형 리모컨이에요(문 잠금·해제용). [근거] Xhorse 상품 사진(대리점 상품 페이지): 키고리가 달린 분리형 리모컨, 구성품에 키날 없음. xhorsetool.com 상품명도 "Hyundai Separate 3 Buttons". (UHS·Keyless City 설명의 "Flip" 표기는 사진과 다름)</t>
         </is>
       </c>
     </row>
@@ -9199,12 +9199,12 @@
       </c>
       <c r="E127" s="8" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>리모컨 키 (키날 따로 끼움)</t>
         </is>
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="G127" s="8" t="inlineStr">
@@ -9236,12 +9236,12 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="N127" s="8" t="n"/>
-      <c r="O127" s="8" t="inlineStr">
-        <is>
-          <t>키날 없이 버튼만 있는 리모컨이에요(문 잠금·해제용). 시동 키가 따로 있는 차에 쓰는 형태라 키날을 끼우지 않아요. [근거] ABKEYS 상품명이 폴딩키("Flip Remote")가 아니라 "Remote Control"이고, 상품 정보에 키날 항목이 없음 (판매처 정보로 본 판단)</t>
-        </is>
-      </c>
+      <c r="N127" s="8" t="inlineStr">
+        <is>
+          <t>Xhorse 상품 사진(대리점 상품 페이지): 구성품 표에 "Key Blade – 별도 구매"로 공용 폴딩 키날 모양 키날이 나옴</t>
+        </is>
+      </c>
+      <c r="O127" s="8" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
@@ -9266,12 +9266,12 @@
       </c>
       <c r="E128" s="8" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>리모컨 키 (키날 따로 끼움)</t>
         </is>
       </c>
       <c r="F128" s="10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="G128" s="8" t="inlineStr">
@@ -9307,12 +9307,12 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="N128" s="8" t="n"/>
-      <c r="O128" s="8" t="inlineStr">
-        <is>
-          <t>키날 없이 버튼만 있는 리모컨으로 판단해요(문 잠금·해제용). [근거] 판매처 상품명에 폴딩(Flip)·키날 표기가 없음 (확인 필요)</t>
-        </is>
-      </c>
+      <c r="N128" s="8" t="inlineStr">
+        <is>
+          <t>XNSZ01EN의 신형 (xhorsestore.co.uk "Second Generation") / Xhorse 상품 사진(대리점 상품 페이지): 구성품 표에 "Key Blade – 별도 구매"로 공용 폴딩 키날 모양 키날이 나옴</t>
+        </is>
+      </c>
+      <c r="O128" s="8" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
@@ -9340,7 +9340,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F129" s="13" t="inlineStr">
+      <c r="F129" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9407,7 +9407,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F130" s="13" t="inlineStr">
+      <c r="F130" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9470,7 +9470,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F131" s="13" t="inlineStr">
+      <c r="F131" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9533,7 +9533,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F132" s="13" t="inlineStr">
+      <c r="F132" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9600,7 +9600,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F133" s="13" t="inlineStr">
+      <c r="F133" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9663,7 +9663,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F134" s="13" t="inlineStr">
+      <c r="F134" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9734,7 +9734,7 @@
           <t>벤츠 키 기판 (BE Key)</t>
         </is>
       </c>
-      <c r="F135" s="10" t="inlineStr">
+      <c r="F135" s="13" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -9801,7 +9801,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F136" s="13" t="inlineStr">
+      <c r="F136" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9864,7 +9864,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F137" s="13" t="inlineStr">
+      <c r="F137" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9931,7 +9931,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F138" s="13" t="inlineStr">
+      <c r="F138" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -9998,7 +9998,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F139" s="13" t="inlineStr">
+      <c r="F139" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10065,7 +10065,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F140" s="13" t="inlineStr">
+      <c r="F140" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10128,7 +10128,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F141" s="13" t="inlineStr">
+      <c r="F141" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10191,7 +10191,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F142" s="13" t="inlineStr">
+      <c r="F142" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10258,7 +10258,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F143" s="13" t="inlineStr">
+      <c r="F143" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10329,7 +10329,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F144" s="13" t="inlineStr">
+      <c r="F144" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10396,7 +10396,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F145" s="13" t="inlineStr">
+      <c r="F145" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10463,7 +10463,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F146" s="13" t="inlineStr">
+      <c r="F146" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10530,7 +10530,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F147" s="13" t="inlineStr">
+      <c r="F147" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10597,7 +10597,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F148" s="13" t="inlineStr">
+      <c r="F148" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10664,7 +10664,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F149" s="13" t="inlineStr">
+      <c r="F149" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10731,7 +10731,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F150" s="13" t="inlineStr">
+      <c r="F150" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10798,7 +10798,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F151" s="13" t="inlineStr">
+      <c r="F151" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -10865,7 +10865,7 @@
           <t>벤츠 키 기판 (BE Key)</t>
         </is>
       </c>
-      <c r="F152" s="10" t="inlineStr">
+      <c r="F152" s="13" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -10932,7 +10932,7 @@
           <t>벤츠 키 기판 (BE Key)</t>
         </is>
       </c>
-      <c r="F153" s="10" t="inlineStr">
+      <c r="F153" s="13" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -10996,12 +10996,12 @@
       </c>
       <c r="E154" s="8" t="inlineStr">
         <is>
-          <t>리모컨</t>
+          <t>폴딩키</t>
         </is>
       </c>
       <c r="F154" s="10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="G154" s="8" t="inlineStr">
@@ -11037,12 +11037,12 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="N154" s="8" t="n"/>
-      <c r="O154" s="8" t="inlineStr">
-        <is>
-          <t>키날 없이 버튼만 있는 리모컨으로 판단해요(문 잠금·해제용). [근거] 판매처 상품명에 폴딩(Flip)·키날 표기가 없음 (확인 필요)</t>
-        </is>
-      </c>
+      <c r="N154" s="8" t="inlineStr">
+        <is>
+          <t>Xhorse 상품 사진(대리점 상품 페이지): 포드 스타일 폴딩키</t>
+        </is>
+      </c>
+      <c r="O154" s="8" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="8" t="inlineStr">
@@ -11070,7 +11070,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F155" s="13" t="inlineStr">
+      <c r="F155" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -11133,7 +11133,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F156" s="13" t="inlineStr">
+      <c r="F156" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -11204,7 +11204,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F157" s="13" t="inlineStr">
+      <c r="F157" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -11275,7 +11275,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F158" s="13" t="inlineStr">
+      <c r="F158" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -11342,7 +11342,7 @@
           <t>폴딩키</t>
         </is>
       </c>
-      <c r="F159" s="13" t="inlineStr">
+      <c r="F159" s="10" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -11546,7 +11546,7 @@
       </c>
       <c r="G162" s="14" t="inlineStr">
         <is>
-          <t>슈퍼칩 (판매처가 XT27A/XT27B/XT57B 구분 안 함)</t>
+          <t>슈퍼칩 (Xhorse 사양표·판매처 모두 "Transponder: yes"만 표기, XT27/XT57 구분 없음)</t>
         </is>
       </c>
       <c r="H162" s="14" t="inlineStr">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="G163" s="14" t="inlineStr">
         <is>
-          <t>슈퍼칩 (판매처가 XT27A/XT27B/XT57B 구분 안 함)</t>
+          <t>슈퍼칩 (Xhorse 사양표·판매처 모두 "Transponder: yes"만 표기, XT27/XT57 구분 없음)</t>
         </is>
       </c>
       <c r="H163" s="14" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="N163" s="14" t="inlineStr">
         <is>
-          <t>형태 판단: keydirect.ca 상품명 "2nd Generation 3-Button Universal Super Remote Flip Key … XEDM24EN" (판매처 상품명에 폴딩 표기 없어 같은 계열 기준으로 판단)</t>
+          <t>Xhorse 상품 사진(대리점 상품 페이지): MQB 폴딩키, 구성품 표에 "Key Blade – 별도 구매" (keydirect.ca 상품명도 "Flip Key")</t>
         </is>
       </c>
       <c r="O163" s="14" t="n"/>
@@ -12287,7 +12287,7 @@
       </c>
       <c r="G173" s="14" t="inlineStr">
         <is>
-          <t>슈퍼칩 (판매처가 XT27A/XT27B/XT57B 구분 안 함)</t>
+          <t>슈퍼칩 (Xhorse 사양표·판매처 모두 "Transponder: yes"만 표기, XT27/XT57 구분 없음)</t>
         </is>
       </c>
       <c r="H173" s="14" t="inlineStr">
@@ -12421,7 +12421,7 @@
       </c>
       <c r="G175" s="14" t="inlineStr">
         <is>
-          <t>슈퍼칩 (판매처가 XT27A/XT27B/XT57B 구분 안 함)</t>
+          <t>슈퍼칩 (Xhorse 사양표·판매처 모두 "Transponder: yes"만 표기, XT27/XT57 구분 없음)</t>
         </is>
       </c>
       <c r="H175" s="14" t="inlineStr">
@@ -12618,7 +12618,7 @@
       </c>
       <c r="G178" s="14" t="inlineStr">
         <is>
-          <t>슈퍼칩 (판매처가 XT27A/XT27B/XT57B 구분 안 함)</t>
+          <t>슈퍼칩 (Xhorse 사양표·판매처 모두 "Transponder: yes"만 표기, XT27/XT57 구분 없음)</t>
         </is>
       </c>
       <c r="H178" s="14" t="inlineStr">
@@ -12986,7 +12986,7 @@
       </c>
       <c r="N183" s="20" t="inlineStr">
         <is>
-          <t>XSMQB1EN의 신형 / xhorseshop.eu: "Blade: Flip HU66 profile blade (Not included)"</t>
+          <t>XSMQB1EN의 신형 / Xhorse 상품 사진(대리점 상품 페이지): MQB 폴딩 스마트키, 구성품 표에 "Key Blade – 별도 구매" (xhorseshop.eu: "Flip HU66 profile blade (Not included)")</t>
         </is>
       </c>
       <c r="O183" s="20" t="n"/>
@@ -13619,7 +13619,7 @@
       </c>
       <c r="G193" s="20" t="inlineStr">
         <is>
-          <t>XM38</t>
+          <t>XM38 (Xhorse 출시 이미지 표기)</t>
         </is>
       </c>
       <c r="H193" s="20" t="inlineStr">
@@ -13649,7 +13649,7 @@
       <c r="N193" s="20" t="n"/>
       <c r="O193" s="20" t="inlineStr">
         <is>
-          <t>판매처에서 비상키 정보를 찾지 못했어요 (벤츠 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
+          <t>비상키 자리는 있고 키날은 따로 사야 해요. 공용 폴딩 키날이 맞는지는 판매처·Xhorse 모두 적지 않았어요 (확인 필요). [근거] Xhorse 상품 사진(대리점 상품 페이지): 구성품 표에 "Key Blade – 별도 구매"(비상키 머리 부품), Best Key Supply "Blade: Not Included"</t>
         </is>
       </c>
     </row>
@@ -13816,12 +13816,12 @@
       </c>
       <c r="G196" s="20" t="inlineStr">
         <is>
-          <t>미기재 (XSCL01EN의 신형)</t>
+          <t>미기재 (XSCL01EN의 신형) – Xhorse 사양표는 "Transponder: NO", UHS·Royal Key Supply는 "Proximity" 표기로 서로 다름</t>
         </is>
       </c>
       <c r="H196" s="20" t="inlineStr">
         <is>
-          <t>미기재 (판매처 7곳 확인, 칩 목록 없음)</t>
+          <t>미기재 (판매처 7곳·Xhorse 사양표 확인, 칩 목록 없음)</t>
         </is>
       </c>
       <c r="I196" s="23" t="n">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="N196" s="20" t="inlineStr">
         <is>
-          <t>XSCL01EN의 신형</t>
+          <t>XSCL01EN의 신형 / Xhorse 상품 사진(대리점 상품 페이지): 구성품 표에 "Key Blade – 별도 구매" (공용 폴딩 키날 모양)</t>
         </is>
       </c>
       <c r="O196" s="20" t="n"/>
@@ -14135,7 +14135,7 @@
       </c>
       <c r="G201" s="20" t="inlineStr">
         <is>
-          <t>XM38</t>
+          <t>XM38 (Xhorse 출시 이미지 표기)</t>
         </is>
       </c>
       <c r="H201" s="20" t="inlineStr">
@@ -14165,7 +14165,7 @@
       <c r="N201" s="20" t="n"/>
       <c r="O201" s="20" t="inlineStr">
         <is>
-          <t>판매처에서 비상키 정보를 찾지 못했어요 (기아 EV 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
+          <t>비상키 자리는 있고 키날은 따로 사야 해요. 공용 폴딩 키날이 맞는지는 판매처·Xhorse 모두 적지 않았어요 (확인 필요). [근거] Xhorse 상품 사진(대리점 상품 페이지): 구성품 표에 "Key Blade – 별도 구매"(비상키 머리 부품), Best Key Supply "Blade: Not Included"</t>
         </is>
       </c>
     </row>
@@ -14202,7 +14202,7 @@
       </c>
       <c r="G202" s="20" t="inlineStr">
         <is>
-          <t>XM38</t>
+          <t>XM38 (Xhorse 출시 이미지 표기)</t>
         </is>
       </c>
       <c r="H202" s="20" t="inlineStr">
@@ -14232,14 +14232,14 @@
       <c r="N202" s="20" t="n"/>
       <c r="O202" s="20" t="inlineStr">
         <is>
-          <t>판매처에서 비상키 정보를 찾지 못했어요 (기아 EV 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
+          <t>비상키 자리는 있고 키날은 따로 사야 해요. 공용 폴딩 키날이 맞는지는 판매처·Xhorse 모두 적지 않았어요 (확인 필요). [근거] Xhorse 상품 사진(대리점 상품 페이지): 구성품 표에 "Key Blade – 별도 구매"(비상키 머리 부품), Best Key Supply "Blade: Not Included"</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="20" t="inlineStr">
         <is>
-          <t>XS 스마트키</t>
+          <t>XS 스마트키 (카드키)</t>
         </is>
       </c>
       <c r="B203" s="21" t="inlineStr">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="E203" s="20" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>카드형 스마트키</t>
         </is>
       </c>
       <c r="F203" s="22" t="inlineStr">
@@ -14306,7 +14306,7 @@
     <row r="204">
       <c r="A204" s="20" t="inlineStr">
         <is>
-          <t>XS 스마트키</t>
+          <t>XS 스마트키 (카드키)</t>
         </is>
       </c>
       <c r="B204" s="21" t="inlineStr">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="E204" s="20" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>카드형 스마트키</t>
         </is>
       </c>
       <c r="F204" s="22" t="inlineStr">
@@ -14730,7 +14730,7 @@
       </c>
       <c r="G210" s="20" t="inlineStr">
         <is>
-          <t>XM38</t>
+          <t>XM38 (Xhorse 출시 이미지 표기)</t>
         </is>
       </c>
       <c r="H210" s="20" t="inlineStr">
@@ -14760,7 +14760,7 @@
       <c r="N210" s="20" t="n"/>
       <c r="O210" s="20" t="inlineStr">
         <is>
-          <t>판매처에서 비상키 정보를 찾지 못했어요 (마세라티 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
+          <t>비상키 자리는 있고 키날은 따로 사야 해요. 공용 폴딩 키날이 맞는지는 판매처·Xhorse 모두 적지 않았어요 (확인 필요). [근거] Xhorse 상품 사진(대리점 상품 페이지): 구성품 표에 "Key Blade – 별도 구매"(비상키 머리 부품), Best Key Supply "Blade: Not Included"</t>
         </is>
       </c>
     </row>
@@ -15180,9 +15180,9 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F217" s="22" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F217" s="25" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G217" s="20" t="inlineStr">
@@ -15214,12 +15214,12 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="N217" s="20" t="n"/>
-      <c r="O217" s="20" t="inlineStr">
-        <is>
-          <t>랜드로버 스마트키 모양이라 랜드로버 스마트키용 비상키(HU101 규격)를 끼우는 것으로 보여요. [근거] ABKEYS가 "Range Rover, Land Rover 2010+ Smart Key Blade, HU101"을 지정, 3D Group도 "Blade Reference HU101". 단 key4는 공용 폴딩 키날 구매를 안내해서 판매처마다 말이 달라요 → 구매 전 확인 필요</t>
-        </is>
-      </c>
+      <c r="N217" s="20" t="inlineStr">
+        <is>
+          <t>Xhorse 상품 사진(대리점 상품 페이지): 구성품 표에 "Key Blade – 별도 구매"로 공용 폴딩 키날 모양 키날이 나옴. 참고: ABKEYS는 HU101 랜드로버 스마트키 비상키를 지정</t>
+        </is>
+      </c>
+      <c r="O217" s="20" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="20" t="inlineStr">
@@ -15247,9 +15247,9 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="F218" s="22" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="F218" s="25" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G218" s="20" t="inlineStr">
@@ -15281,12 +15281,12 @@
           <t>링크</t>
         </is>
       </c>
-      <c r="N218" s="20" t="n"/>
-      <c r="O218" s="20" t="inlineStr">
-        <is>
-          <t>키날 정보를 적은 판매처를 찾지 못했어요. [근거] Locksmith Keyless 등 설명에 키날 언급 없음. 같은 랜드로버 모양(XSLR01EN)은 ABKEYS가 랜드로버 스마트키용 비상키(HU101)를 지정 → 같은 방식일 가능성이 높지만 확인 필요</t>
-        </is>
-      </c>
+      <c r="N218" s="20" t="inlineStr">
+        <is>
+          <t>형태 판단: 같은 랜드로버 모양 XSLR01EN의 Xhorse 구성품 사진에 공용 폴딩 키날 모양 "Key Blade – 별도 구매". XSLR03EN은 Best Key Supply·Locksmith Keyless "Blade: Not Included"</t>
+        </is>
+      </c>
+      <c r="O218" s="20" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="20" t="inlineStr">
@@ -15489,7 +15489,7 @@
       <c r="N221" s="20" t="n"/>
       <c r="O221" s="20" t="inlineStr">
         <is>
-          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
+          <t>손목시계형 스마트키라 키날을 끼우는 자리가 없어요. [근거] 판매처 상품명 "Smart Watch Wearable Super Car Key"</t>
         </is>
       </c>
     </row>
@@ -15556,7 +15556,7 @@
       <c r="N222" s="20" t="n"/>
       <c r="O222" s="20" t="inlineStr">
         <is>
-          <t>휴대폰 디지털키·손목시계형 키라 키날을 끼우는 자리가 없어요. [근거] ABKEYS 상품명 "Bluetooth Digital Smart Key" / "Smart Watch Wearable Car Key"</t>
+          <t>손목시계형 스마트키라 키날을 끼우는 자리가 없어요. [근거] 판매처 상품명 "Smart Watch Wearable Super Car Key"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add XT/XM chip family section to PDF; align XT27A/XT27B lists with Xhorse comparison
Explains that XT super chips and XM smart-key chips are separate
families, lists each chip's definition and full support range, and moves
47/49 from XT27A to XT27B per the Xhorse user-guide comparison table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_모델별_가격표.xlsx
+++ b/Xhorse_모델별_가격표.xlsx
@@ -11417,7 +11417,7 @@
       </c>
       <c r="H160" s="14" t="inlineStr">
         <is>
-          <t>11, 12, 13, 7935, 7936, 46, 47, 48, 49, 4A, 4C, 4D, 4E, 8A, 8C, 8E, MQB48</t>
+          <t>11, 12, 13, 7935, 46 (7936 등), 48, 4C, 4D, 4E, 8A, 8C, 8E + 47, 49, 4A, MQB48 (XT27B에서 추가)</t>
         </is>
       </c>
       <c r="I160" s="17" t="n">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="H164" s="14" t="inlineStr">
         <is>
-          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
+          <t>11·12·13, 7935 (33·40~44), 46 (7936·7937·7946), 48, 4C, 4D, 4E, 8A, 8C, 8E (47·49는 Xhorse 비교표상 XT27B부터, 일부 판매처는 XT27A에도 표기)</t>
         </is>
       </c>
       <c r="I164" s="17" t="n">
@@ -11819,7 +11819,7 @@
       </c>
       <c r="H166" s="14" t="inlineStr">
         <is>
-          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
+          <t>11·12·13, 7935 (33·40~44), 46 (7936·7937·7946), 48, 4C, 4D, 4E, 8A, 8C, 8E (47·49는 Xhorse 비교표상 XT27B부터, 일부 판매처는 XT27A에도 표기)</t>
         </is>
       </c>
       <c r="I166" s="17" t="n">
@@ -11957,7 +11957,7 @@
       </c>
       <c r="H168" s="14" t="inlineStr">
         <is>
-          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
+          <t>11·12·13, 7935 (33·40~44), 46 (7936·7937·7946), 48, 4C, 4D, 4E, 8A, 8C, 8E (47·49는 Xhorse 비교표상 XT27B부터, 일부 판매처는 XT27A에도 표기)</t>
         </is>
       </c>
       <c r="I168" s="17" t="n">
@@ -12020,7 +12020,7 @@
       </c>
       <c r="H169" s="14" t="inlineStr">
         <is>
-          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
+          <t>11·12·13, 7935 (33·40~44), 46 (7936·7937·7946), 48, 4C, 4D, 4E, 8A, 8C, 8E (47·49는 Xhorse 비교표상 XT27B부터, 일부 판매처는 XT27A에도 표기)</t>
         </is>
       </c>
       <c r="I169" s="17" t="n">
@@ -12087,7 +12087,7 @@
       </c>
       <c r="H170" s="14" t="inlineStr">
         <is>
-          <t>11, 12, 13, 7935, 7936, 46, 47, 48, 49, 4A, 4C, 4D, 4E, 8A, 8C, 8E, MQB48</t>
+          <t>11, 12, 13, 7935, 46 (7936 등), 48, 4C, 4D, 4E, 8A, 8C, 8E + 47, 49, 4A, MQB48 (XT27B에서 추가)</t>
         </is>
       </c>
       <c r="I170" s="17" t="n">
@@ -12225,7 +12225,7 @@
       </c>
       <c r="H172" s="14" t="inlineStr">
         <is>
-          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
+          <t>11·12·13, 7935 (33·40~44), 46 (7936·7937·7946), 48, 4C, 4D, 4E, 8A, 8C, 8E (47·49는 Xhorse 비교표상 XT27B부터, 일부 판매처는 XT27A에도 표기)</t>
         </is>
       </c>
       <c r="I172" s="17" t="n">
@@ -12359,7 +12359,7 @@
       </c>
       <c r="H174" s="14" t="inlineStr">
         <is>
-          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13</t>
+          <t>11·12·13, 7935 (33·40~44), 46 (7936·7937·7946), 48, 4C, 4D, 4E, 8A, 8C, 8E (47·49는 Xhorse 비교표상 XT27B부터, 일부 판매처는 XT27A에도 표기)</t>
         </is>
       </c>
       <c r="I174" s="17" t="n">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="H176" s="14" t="inlineStr">
         <is>
-          <t>7935 (33·40~44), 7936·7937·7946 (46), 7938·7947 (47), 7939 (49), 4D, 4E, 4C, 8C, 8A, 48, 8E, 11·12·13 (XT57B 제품이면 XT57B 목록)</t>
+          <t>11·12·13, 7935 (33·40~44), 46 (7936·7937·7946), 48, 4C, 4D, 4E, 8A, 8C, 8E (47·49는 Xhorse 비교표상 XT27B부터, 일부 판매처는 XT27A에도 표기) (XT57B 제품이면 XT57B 목록)</t>
         </is>
       </c>
       <c r="I176" s="17" t="n">

</xml_diff>